<commit_message>
Delete lots of duplicate files
</commit_message>
<xml_diff>
--- a/Voltage_discharge.xlsx
+++ b/Voltage_discharge.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="36" windowWidth="15960" windowHeight="13176" firstSheet="2" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="36" windowWidth="15960" windowHeight="13176" firstSheet="2" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Export Summary" sheetId="1" r:id="rId1"/>
@@ -12,6 +12,7 @@
     <sheet name="Sheet 1-1 - 12V 10Ah LFP Discha" sheetId="3" r:id="rId3"/>
     <sheet name="Solar Panel Comparisons - Solar" sheetId="4" r:id="rId4"/>
     <sheet name="Riemann Sum - Midpoint Riemann " sheetId="5" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="125725"/>
 </workbook>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="38">
   <si>
     <t>This document was exported from Numbers.  Each table was converted to an Excel worksheet. All other objects on each Numbers sheet were placed on separate worksheets. Please be aware that formula calculations may differ in Excel.</t>
   </si>
@@ -141,16 +142,26 @@
     <t>Current by Solar</t>
   </si>
   <si>
-    <t>Current by Solar (Tracker Off)</t>
+    <t>Dual Axis</t>
   </si>
   <si>
-    <t>Current by Solar (Tracker On)</t>
+    <r>
+      <t>Fixed at 29</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t xml:space="preserve"> Degrees</t>
+    </r>
   </si>
   <si>
-    <t>Average * Time (Tracker Off)</t>
+    <t>Single Axis</t>
   </si>
   <si>
-    <t>Average * Time (Tracker On)</t>
+    <t>AVERAGES</t>
   </si>
   <si>
     <t>SUM</t>
@@ -160,7 +171,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -198,6 +209,11 @@
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Helvetica"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="8"/>
+      <name val="Helvetica Neue"/>
     </font>
   </fonts>
   <fills count="6">
@@ -351,7 +367,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -460,6 +476,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -469,6 +488,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="18" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="18" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -477,15 +514,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="18" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="18" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -576,9 +604,9 @@
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
           <c:x val="9.1001100000000015E-2"/>
-          <c:y val="0.12368000000000008"/>
+          <c:y val="0.12368000000000012"/>
           <c:w val="0.89403199999999949"/>
-          <c:h val="0.81033699999999931"/>
+          <c:h val="0.81033699999999853"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -1851,11 +1879,11 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="176166784"/>
-        <c:axId val="176256128"/>
+        <c:axId val="165505280"/>
+        <c:axId val="165565952"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="176166784"/>
+        <c:axId val="165505280"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1887,14 +1915,14 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="176256128"/>
+        <c:crossAx val="165565952"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
         <c:minorUnit val="0.5"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="176256128"/>
+        <c:axId val="165565952"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="13"/>
@@ -1937,7 +1965,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="176166784"/>
+        <c:crossAx val="165505280"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="0.25"/>
@@ -1961,7 +1989,7 @@
           <c:x val="7.5607700000000014E-2"/>
           <c:y val="0"/>
           <c:w val="0.88914199999999999"/>
-          <c:h val="6.4066700000000101E-2"/>
+          <c:h val="6.4066700000000185E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -2001,7 +2029,7 @@
   </c:spPr>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000056" l="0.70000000000000051" r="0.70000000000000051" t="0.75000000000000056" header="0.30000000000000027" footer="0.30000000000000027"/>
+    <c:pageMargins b="0.75000000000000133" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000133" header="0.30000000000000032" footer="0.30000000000000032"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -2019,9 +2047,9 @@
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
           <c:x val="9.1001100000000015E-2"/>
-          <c:y val="0.12368000000000008"/>
+          <c:y val="0.12368000000000012"/>
           <c:w val="0.89403199999999949"/>
-          <c:h val="0.81033699999999931"/>
+          <c:h val="0.81033699999999853"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -3460,11 +3488,11 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="202030080"/>
-        <c:axId val="175948544"/>
+        <c:axId val="165210752"/>
+        <c:axId val="165228928"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="202030080"/>
+        <c:axId val="165210752"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3496,14 +3524,14 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="175948544"/>
+        <c:crossAx val="165228928"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
         <c:minorUnit val="0.5"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="175948544"/>
+        <c:axId val="165228928"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="13"/>
@@ -3546,7 +3574,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="202030080"/>
+        <c:crossAx val="165210752"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="0.25"/>
@@ -3570,7 +3598,7 @@
           <c:x val="7.5607700000000014E-2"/>
           <c:y val="0"/>
           <c:w val="0.88914199999999999"/>
-          <c:h val="6.4066700000000101E-2"/>
+          <c:h val="6.4066700000000185E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -3610,7 +3638,7 @@
   </c:spPr>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000056" l="0.70000000000000051" r="0.70000000000000051" t="0.75000000000000056" header="0.30000000000000027" footer="0.30000000000000027"/>
+    <c:pageMargins b="0.75000000000000133" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000133" header="0.30000000000000032" footer="0.30000000000000032"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -3628,9 +3656,9 @@
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
           <c:x val="9.1082899999999994E-2"/>
-          <c:y val="0.12368000000000008"/>
+          <c:y val="0.12368000000000012"/>
           <c:w val="0.89393599999999951"/>
-          <c:h val="0.81033699999999931"/>
+          <c:h val="0.81033699999999853"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -4572,11 +4600,11 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="176157056"/>
-        <c:axId val="176158592"/>
+        <c:axId val="165306368"/>
+        <c:axId val="165307904"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="176157056"/>
+        <c:axId val="165306368"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4608,14 +4636,14 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="176158592"/>
+        <c:crossAx val="165307904"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="3"/>
         <c:minorUnit val="1.5"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="176158592"/>
+        <c:axId val="165307904"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="13"/>
@@ -4657,7 +4685,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="176157056"/>
+        <c:crossAx val="165306368"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="0.25"/>
@@ -4681,7 +4709,7 @@
           <c:x val="7.5226400000000082E-2"/>
           <c:y val="0"/>
           <c:w val="0.88994100000000065"/>
-          <c:h val="6.4066700000000101E-2"/>
+          <c:h val="6.4066700000000185E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -4721,7 +4749,7 @@
   </c:spPr>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000056" l="0.70000000000000051" r="0.70000000000000051" t="0.75000000000000056" header="0.30000000000000027" footer="0.30000000000000027"/>
+    <c:pageMargins b="0.75000000000000133" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000133" header="0.30000000000000032" footer="0.30000000000000032"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -4739,9 +4767,9 @@
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
           <c:x val="9.1001100000000015E-2"/>
-          <c:y val="0.12368000000000008"/>
+          <c:y val="0.12368000000000012"/>
           <c:w val="0.89403199999999949"/>
-          <c:h val="0.81033699999999931"/>
+          <c:h val="0.81033699999999853"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -6014,11 +6042,11 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="176191360"/>
-        <c:axId val="176192896"/>
+        <c:axId val="165340672"/>
+        <c:axId val="165342208"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="176191360"/>
+        <c:axId val="165340672"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6050,14 +6078,14 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="176192896"/>
+        <c:crossAx val="165342208"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
         <c:minorUnit val="0.5"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="176192896"/>
+        <c:axId val="165342208"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="13"/>
@@ -6100,7 +6128,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="176191360"/>
+        <c:crossAx val="165340672"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="0.25"/>
@@ -6124,7 +6152,7 @@
           <c:x val="7.5607700000000014E-2"/>
           <c:y val="0"/>
           <c:w val="0.88914199999999999"/>
-          <c:h val="6.4066700000000101E-2"/>
+          <c:h val="6.4066700000000185E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -6164,7 +6192,7 @@
   </c:spPr>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000056" l="0.70000000000000051" r="0.70000000000000051" t="0.75000000000000056" header="0.30000000000000027" footer="0.30000000000000027"/>
+    <c:pageMargins b="0.75000000000000133" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000133" header="0.30000000000000032" footer="0.30000000000000032"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -6181,10 +6209,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="6.4312400000000103E-2"/>
-          <c:y val="0.12368000000000008"/>
+          <c:x val="6.4312400000000242E-2"/>
+          <c:y val="0.12368000000000012"/>
           <c:w val="0.88765000000000005"/>
-          <c:h val="0.81033699999999931"/>
+          <c:h val="0.81033699999999853"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -6392,11 +6420,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="176303104"/>
-        <c:axId val="176308992"/>
+        <c:axId val="165501568"/>
+        <c:axId val="165527936"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="176303104"/>
+        <c:axId val="165501568"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="806395000"/>
@@ -6429,12 +6457,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="176308992"/>
+        <c:crossAx val="165527936"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="176308992"/>
+        <c:axId val="165527936"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6475,7 +6503,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="176303104"/>
+        <c:crossAx val="165501568"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="0.2"/>
@@ -6499,7 +6527,7 @@
           <c:x val="4.0081200000000004E-2"/>
           <c:y val="0"/>
           <c:w val="0.9"/>
-          <c:h val="6.4066700000000101E-2"/>
+          <c:h val="6.4066700000000185E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -6539,7 +6567,680 @@
   </c:spPr>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000056" l="0.70000000000000051" r="0.70000000000000051" t="0.75000000000000056" header="0.30000000000000027" footer="0.30000000000000027"/>
+    <c:pageMargins b="0.75000000000000133" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000133" header="0.30000000000000032" footer="0.30000000000000032"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Current Production</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> over Time</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Fixed at 29 Degrees</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet1!$A$2:$A$27</c:f>
+              <c:numCache>
+                <c:formatCode>h:mm\ AM/PM</c:formatCode>
+                <c:ptCount val="26"/>
+                <c:pt idx="0">
+                  <c:v>46225.28125</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46225.302083333336</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46225.322916666664</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>46225.34375</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>46225.364583333336</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>46225.385416666664</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>46225.40625</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>46225.427083333336</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>46225.447916666664</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>46225.46875</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>46225.489583333336</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>46225.510416666664</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>46225.53125</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>46225.552083333336</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>46225.572916666664</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>46225.59375</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>46225.614583333336</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>46225.635416666664</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>46225.65625</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>46225.677083333336</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>46225.697916666664</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>46225.71875</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>46225.739583333336</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>46225.760416666664</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.78125</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.80208333333333337</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$B$2:$B$27</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="26"/>
+                <c:pt idx="0">
+                  <c:v>5.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.03</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.13</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.23</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.37</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.49</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.87</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.93</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.98</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.99</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.99</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.97</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.93</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.88</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.83</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.75</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.64</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.53</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.36</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.28000000000000003</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.16</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.05</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.01</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Single Axis</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet1!$A$2:$A$27</c:f>
+              <c:numCache>
+                <c:formatCode>h:mm\ AM/PM</c:formatCode>
+                <c:ptCount val="26"/>
+                <c:pt idx="0">
+                  <c:v>46225.28125</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46225.302083333336</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46225.322916666664</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>46225.34375</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>46225.364583333336</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>46225.385416666664</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>46225.40625</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>46225.427083333336</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>46225.447916666664</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>46225.46875</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>46225.489583333336</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>46225.510416666664</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>46225.53125</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>46225.552083333336</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>46225.572916666664</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>46225.59375</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>46225.614583333336</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>46225.635416666664</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>46225.65625</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>46225.677083333336</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>46225.697916666664</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>46225.71875</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>46225.739583333336</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>46225.760416666664</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.78125</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.80208333333333337</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$C$2:$C$27</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="26"/>
+                <c:pt idx="0">
+                  <c:v>0.23</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.67</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.77</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.85</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.89</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.94</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.96</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.98</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.99</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.98</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.99</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.99</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.99</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.98</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.95</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.93</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.89</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.89</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.84</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.74</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.6</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$D$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Dual Axis</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet1!$A$2:$A$27</c:f>
+              <c:numCache>
+                <c:formatCode>h:mm\ AM/PM</c:formatCode>
+                <c:ptCount val="26"/>
+                <c:pt idx="0">
+                  <c:v>46225.28125</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46225.302083333336</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46225.322916666664</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>46225.34375</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>46225.364583333336</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>46225.385416666664</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>46225.40625</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>46225.427083333336</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>46225.447916666664</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>46225.46875</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>46225.489583333336</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>46225.510416666664</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>46225.53125</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>46225.552083333336</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>46225.572916666664</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>46225.59375</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>46225.614583333336</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>46225.635416666664</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>46225.65625</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>46225.677083333336</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>46225.697916666664</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>46225.71875</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>46225.739583333336</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>46225.760416666664</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.78125</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.80208333333333337</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$D$2:$D$27</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="26"/>
+                <c:pt idx="0">
+                  <c:v>0.35</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.55000000000000004</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.74</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.84</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.86</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.9</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.93</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.96</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.99</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.02</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.03</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.03</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.03</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.02</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1.01</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.97</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.97</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.95</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.92</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.88</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.86</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.87</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.78</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.62</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.41</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:marker val="1"/>
+        <c:axId val="165717504"/>
+        <c:axId val="165719040"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="165717504"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="h:mm\ AM/PM" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="165719040"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="165719040"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Solar Current (A)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="165717504"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75000000000000089" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000089" header="0.30000000000000032" footer="0.30000000000000032"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -6693,6 +7394,41 @@
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="8" name="Scatter Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>433386</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>147638</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>464819</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -7760,11 +8496,11 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:4" ht="49.95" customHeight="1">
-      <c r="B3" s="39" t="s">
+      <c r="B3" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
     </row>
     <row r="7" spans="2:4" ht="17.399999999999999">
       <c r="B7" s="1" t="s">
@@ -7865,17 +8601,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="27.75" customHeight="1">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="41"/>
-      <c r="I1" s="41"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
     </row>
     <row r="2" spans="1:9" ht="20.55" customHeight="1">
       <c r="A2" s="6"/>
@@ -12040,15 +12776,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="27.75" customHeight="1">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
     </row>
     <row r="2" spans="1:7" ht="20.55" customHeight="1">
       <c r="A2" s="6"/>
@@ -15913,15 +16649,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="27.75" customHeight="1">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="48" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
     </row>
     <row r="2" spans="1:7" ht="20.55" customHeight="1">
       <c r="A2" s="21"/>
@@ -15937,9 +16673,7 @@
       <c r="E2" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="21" t="s">
-        <v>32</v>
-      </c>
+      <c r="F2" s="21"/>
       <c r="G2" s="21"/>
     </row>
     <row r="3" spans="1:7" ht="20.55" customHeight="1">
@@ -15970,9 +16704,7 @@
       <c r="C4" s="29">
         <v>0.59</v>
       </c>
-      <c r="D4" s="42">
-        <v>0.30208333333333331</v>
-      </c>
+      <c r="D4" s="16"/>
       <c r="E4" s="30">
         <v>0.19</v>
       </c>
@@ -15993,9 +16725,7 @@
       <c r="C5" s="29">
         <v>0.47</v>
       </c>
-      <c r="D5" s="25">
-        <v>46223.322916666701</v>
-      </c>
+      <c r="D5" s="16"/>
       <c r="E5" s="30">
         <v>0.68</v>
       </c>
@@ -16016,9 +16746,7 @@
       <c r="C6" s="15">
         <v>0.35</v>
       </c>
-      <c r="D6" s="42">
-        <v>46222.34375</v>
-      </c>
+      <c r="D6" s="16"/>
       <c r="E6" s="30">
         <v>0.57999999999999996</v>
       </c>
@@ -16039,9 +16767,7 @@
       <c r="C7" s="15">
         <v>0.24</v>
       </c>
-      <c r="D7" s="25">
-        <v>46221.364583333299</v>
-      </c>
+      <c r="D7" s="16"/>
       <c r="E7" s="30">
         <v>0.56000000000000005</v>
       </c>
@@ -16062,9 +16788,7 @@
       <c r="C8" s="29">
         <v>0.12</v>
       </c>
-      <c r="D8" s="42">
-        <v>46220.385416666701</v>
-      </c>
+      <c r="D8" s="16"/>
       <c r="E8" s="30">
         <v>0.52</v>
       </c>
@@ -16085,7 +16809,7 @@
       <c r="C9" s="29">
         <v>0.71</v>
       </c>
-      <c r="D9" s="42"/>
+      <c r="D9" s="16"/>
       <c r="E9" s="30"/>
       <c r="F9" s="30"/>
       <c r="G9" s="30"/>
@@ -16098,9 +16822,7 @@
       <c r="C10" s="29">
         <v>0.64</v>
       </c>
-      <c r="D10" s="42">
-        <v>0.40625</v>
-      </c>
+      <c r="D10" s="16"/>
       <c r="E10" s="30">
         <v>0.49</v>
       </c>
@@ -16121,9 +16843,7 @@
       <c r="C11" s="29">
         <v>0.54</v>
       </c>
-      <c r="D11" s="42">
-        <v>0.42708333333333298</v>
-      </c>
+      <c r="D11" s="16"/>
       <c r="E11" s="30">
         <v>0.46</v>
       </c>
@@ -16144,9 +16864,7 @@
       <c r="C12" s="29">
         <v>0.47</v>
       </c>
-      <c r="D12" s="42">
-        <v>0.44791666666666702</v>
-      </c>
+      <c r="D12" s="16"/>
       <c r="E12" s="30">
         <v>0.43</v>
       </c>
@@ -16167,9 +16885,7 @@
       <c r="C13" s="29">
         <v>0.4</v>
       </c>
-      <c r="D13" s="42">
-        <v>0.46875</v>
-      </c>
+      <c r="D13" s="16"/>
       <c r="E13" s="30">
         <v>0.42</v>
       </c>
@@ -16190,9 +16906,7 @@
       <c r="C14" s="29">
         <v>0.36</v>
       </c>
-      <c r="D14" s="42">
-        <v>0.48958333333333398</v>
-      </c>
+      <c r="D14" s="16"/>
       <c r="E14" s="30">
         <v>0.4</v>
       </c>
@@ -16213,9 +16927,7 @@
       <c r="C15" s="29">
         <v>0.34</v>
       </c>
-      <c r="D15" s="42">
-        <v>0.51041666666666696</v>
-      </c>
+      <c r="D15" s="16"/>
       <c r="E15" s="30">
         <v>0.4</v>
       </c>
@@ -16236,9 +16948,7 @@
       <c r="C16" s="29">
         <v>0.32</v>
       </c>
-      <c r="D16" s="42">
-        <v>0.53125</v>
-      </c>
+      <c r="D16" s="16"/>
       <c r="E16" s="30">
         <v>0.39</v>
       </c>
@@ -16259,9 +16969,7 @@
       <c r="C17" s="29">
         <v>0.33</v>
       </c>
-      <c r="D17" s="42">
-        <v>0.55208333333333404</v>
-      </c>
+      <c r="D17" s="16"/>
       <c r="E17" s="30">
         <v>0.39</v>
       </c>
@@ -16282,9 +16990,7 @@
       <c r="C18" s="29">
         <v>0.34</v>
       </c>
-      <c r="D18" s="42">
-        <v>0.57291666666666696</v>
-      </c>
+      <c r="D18" s="16"/>
       <c r="E18" s="30">
         <v>0.4</v>
       </c>
@@ -16305,9 +17011,7 @@
       <c r="C19" s="29">
         <v>0.38</v>
       </c>
-      <c r="D19" s="42">
-        <v>0.59375</v>
-      </c>
+      <c r="D19" s="16"/>
       <c r="E19" s="30">
         <v>0.4</v>
       </c>
@@ -16328,9 +17032,7 @@
       <c r="C20" s="29">
         <v>0.42</v>
       </c>
-      <c r="D20" s="42">
-        <v>0.61458333333333304</v>
-      </c>
+      <c r="D20" s="16"/>
       <c r="E20" s="30">
         <v>0.42</v>
       </c>
@@ -16351,9 +17053,7 @@
       <c r="C21" s="29">
         <v>0.47</v>
       </c>
-      <c r="D21" s="42">
-        <v>0.63541666666666696</v>
-      </c>
+      <c r="D21" s="16"/>
       <c r="E21" s="30">
         <v>0.44</v>
       </c>
@@ -16374,9 +17074,7 @@
       <c r="C22" s="29">
         <v>0.55000000000000004</v>
       </c>
-      <c r="D22" s="42">
-        <v>0.65625</v>
-      </c>
+      <c r="D22" s="16"/>
       <c r="E22" s="30">
         <v>0.46</v>
       </c>
@@ -16397,9 +17095,7 @@
       <c r="C23" s="29">
         <v>0.65</v>
       </c>
-      <c r="D23" s="42">
-        <v>0.67708333333333304</v>
-      </c>
+      <c r="D23" s="16"/>
       <c r="E23" s="30">
         <v>0.48</v>
       </c>
@@ -16420,9 +17116,7 @@
       <c r="C24" s="29">
         <v>0.75</v>
       </c>
-      <c r="D24" s="42">
-        <v>0.69791666666666696</v>
-      </c>
+      <c r="D24" s="16"/>
       <c r="E24" s="30">
         <v>0.52</v>
       </c>
@@ -16443,7 +17137,7 @@
       <c r="C25" s="29">
         <v>0.1</v>
       </c>
-      <c r="D25" s="42"/>
+      <c r="D25" s="16"/>
       <c r="E25" s="30"/>
       <c r="F25" s="30"/>
       <c r="G25" s="30"/>
@@ -16456,9 +17150,7 @@
       <c r="C26" s="29">
         <v>0.2</v>
       </c>
-      <c r="D26" s="42">
-        <v>0.71875</v>
-      </c>
+      <c r="D26" s="16"/>
       <c r="E26" s="30">
         <v>0.56000000000000005</v>
       </c>
@@ -16479,9 +17171,7 @@
       <c r="C27" s="29">
         <v>0.32</v>
       </c>
-      <c r="D27" s="42">
-        <v>0.73958333333333337</v>
-      </c>
+      <c r="D27" s="16"/>
       <c r="E27" s="30">
         <v>0.55000000000000004</v>
       </c>
@@ -16502,9 +17192,7 @@
       <c r="C28" s="29">
         <v>0.45</v>
       </c>
-      <c r="D28" s="42">
-        <v>0.76041666666666663</v>
-      </c>
+      <c r="D28" s="16"/>
       <c r="E28" s="30">
         <v>0.03</v>
       </c>
@@ -16524,17 +17212,12 @@
       <c r="B29" s="28">
         <v>0.78125</v>
       </c>
-      <c r="C29" s="29"/>
-      <c r="D29" s="43">
-        <v>0.78125</v>
-      </c>
-      <c r="E29" s="30">
-        <v>0.19</v>
-      </c>
-      <c r="F29" s="30">
-        <f t="shared" ref="F29:F30" si="3">0.69-E29</f>
-        <v>0.49999999999999994</v>
-      </c>
+      <c r="C29" s="29">
+        <v>4.9024999999999999</v>
+      </c>
+      <c r="D29" s="30"/>
+      <c r="E29" s="30"/>
+      <c r="F29" s="30"/>
       <c r="G29" s="30"/>
     </row>
     <row r="30" spans="1:7" ht="20.399999999999999" customHeight="1">
@@ -16544,17 +17227,12 @@
       <c r="B30" s="28">
         <v>0.80208333333333337</v>
       </c>
-      <c r="C30" s="29"/>
-      <c r="D30" s="43">
-        <v>0.80208333333333337</v>
-      </c>
-      <c r="E30" s="30">
-        <v>0.4</v>
-      </c>
-      <c r="F30" s="30">
-        <f t="shared" si="3"/>
-        <v>0.28999999999999992</v>
-      </c>
+      <c r="C30" s="29">
+        <v>0.69</v>
+      </c>
+      <c r="D30" s="30"/>
+      <c r="E30" s="30"/>
+      <c r="F30" s="30"/>
       <c r="G30" s="30"/>
     </row>
     <row r="31" spans="1:7" ht="20.399999999999999" customHeight="1">
@@ -16614,27 +17292,27 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr defaultColWidth="16.33203125" defaultRowHeight="19.95" customHeight="1"/>
   <cols>
     <col min="1" max="10" width="16.33203125" style="35" customWidth="1"/>
     <col min="11" max="16384" width="16.33203125" style="35"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="27.75" customHeight="1">
-      <c r="A1" s="44" t="s">
+    <row r="1" spans="1:9" ht="27.75" customHeight="1">
+      <c r="A1" s="48" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-    </row>
-    <row r="2" spans="1:10" ht="33" customHeight="1">
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+    </row>
+    <row r="2" spans="1:9" ht="20.25" customHeight="1">
       <c r="A2" s="7" t="s">
         <v>18</v>
       </c>
@@ -16644,866 +17322,662 @@
       <c r="C2" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="36"/>
+      <c r="E2" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="F2" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="G2" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="G2" s="21" t="s">
-        <v>33</v>
-      </c>
       <c r="H2" s="8" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="I2" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="J2" s="8" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="20.55" customHeight="1">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="20.55" customHeight="1">
       <c r="A3" s="23">
         <v>46225.28125</v>
       </c>
-      <c r="B3" s="36">
+      <c r="B3" s="37">
         <v>0.72</v>
       </c>
       <c r="C3" s="12"/>
-      <c r="D3" s="11">
+      <c r="D3" s="12"/>
+      <c r="E3" s="11">
         <v>0.5</v>
       </c>
-      <c r="E3" s="11">
+      <c r="F3" s="11">
         <v>0.69</v>
       </c>
-      <c r="F3" s="11">
+      <c r="G3" s="11">
         <v>1.3</v>
       </c>
-      <c r="G3" s="30">
+      <c r="H3" s="11">
         <v>0</v>
       </c>
-      <c r="H3" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F3</f>
-        <v>0.28999999999999992</v>
-      </c>
       <c r="I3" s="12"/>
     </row>
-    <row r="4" spans="1:10" ht="20.399999999999999" customHeight="1">
+    <row r="4" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A4" s="28">
         <v>46225.302083333336</v>
       </c>
-      <c r="B4" s="37">
+      <c r="B4" s="38">
         <v>0.59</v>
       </c>
       <c r="C4" s="15" cm="1">
-        <f t="array" ref="C4">(B4+B3)/2*$D$3</f>
+        <f t="array" ref="C4">(B4+B3)/2*$E$3</f>
         <v>0.32750000000000001</v>
       </c>
       <c r="D4" s="16"/>
       <c r="E4" s="16"/>
       <c r="F4" s="16"/>
-      <c r="G4" s="30">
-        <f t="shared" ref="G4:G8" si="0">0.69-B4</f>
+      <c r="G4" s="16"/>
+      <c r="H4" s="15" cm="1">
+        <f t="array" ref="H4">-B4+$F$3</f>
         <v>9.9999999999999978E-2</v>
       </c>
-      <c r="H4" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F4</f>
-        <v>0.49999999999999994</v>
-      </c>
-      <c r="I4" s="15">
-        <f>(G4+G3)/2*$D$3</f>
+      <c r="I4" s="15" cm="1">
+        <f t="array" ref="I4">(H4+H3)/2*$E$3</f>
         <v>2.4999999999999994E-2</v>
       </c>
-      <c r="J4" s="35">
-        <f>(H4+H3)/2*$D$3</f>
-        <v>0.19749999999999995</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="20.399999999999999" customHeight="1">
+    </row>
+    <row r="5" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A5" s="28">
         <v>46225.322916666664</v>
       </c>
-      <c r="B5" s="37">
+      <c r="B5" s="38">
         <v>0.47</v>
       </c>
       <c r="C5" s="15" cm="1">
-        <f t="array" ref="C5">(B5+B4)/2*$D$3</f>
+        <f t="array" ref="C5">(B5+B4)/2*$E$3</f>
         <v>0.26500000000000001</v>
       </c>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
       <c r="F5" s="16"/>
-      <c r="G5" s="30">
-        <f t="shared" si="0"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="15" cm="1">
+        <f t="array" ref="H5">-B5+$F$3</f>
         <v>0.21999999999999997</v>
       </c>
-      <c r="H5" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F5</f>
-        <v>0.62</v>
-      </c>
-      <c r="I5" s="15">
-        <f t="shared" ref="I5:I8" si="1">(G5+G4)/2*$D$3</f>
+      <c r="I5" s="15" cm="1">
+        <f t="array" ref="I5">(H5+H4)/2*$E$3</f>
         <v>7.9999999999999988E-2</v>
       </c>
-      <c r="J5" s="35">
-        <f t="shared" ref="J5:J30" si="2">(H5+H4)/2*$D$3</f>
-        <v>0.27999999999999997</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="20.100000000000001" customHeight="1">
+    </row>
+    <row r="6" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A6" s="28">
         <v>46225.34375</v>
       </c>
-      <c r="B6" s="38">
+      <c r="B6" s="39">
         <v>0.35</v>
       </c>
       <c r="C6" s="15" cm="1">
-        <f t="array" ref="C6">(B6+B5)/2*$D$3</f>
+        <f t="array" ref="C6">(B6+B5)/2*$E$3</f>
         <v>0.20499999999999999</v>
       </c>
       <c r="D6" s="16"/>
       <c r="E6" s="16"/>
       <c r="F6" s="16"/>
-      <c r="G6" s="30">
-        <f t="shared" si="0"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="15" cm="1">
+        <f t="array" ref="H6">-B6+$F$3</f>
         <v>0.33999999999999997</v>
       </c>
-      <c r="H6" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F6</f>
-        <v>0.72000000000000008</v>
-      </c>
-      <c r="I6" s="15">
-        <f t="shared" si="1"/>
+      <c r="I6" s="15" cm="1">
+        <f t="array" ref="I6">(H6+H5)/2*$E$3</f>
         <v>0.13999999999999999</v>
       </c>
-      <c r="J6" s="35">
-        <f t="shared" si="2"/>
-        <v>0.33500000000000002</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="20.100000000000001" customHeight="1">
+    </row>
+    <row r="7" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A7" s="28">
         <v>46225.364583333336</v>
       </c>
-      <c r="B7" s="38">
+      <c r="B7" s="39">
         <v>0.24</v>
       </c>
       <c r="C7" s="15" cm="1">
-        <f t="array" ref="C7">(B7+B6)/2*$D$3</f>
+        <f t="array" ref="C7">(B7+B6)/2*$E$3</f>
         <v>0.14749999999999999</v>
       </c>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
-      <c r="G7" s="30">
-        <f t="shared" si="0"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="15" cm="1">
+        <f t="array" ref="H7">-B7+$F$3</f>
         <v>0.44999999999999996</v>
       </c>
-      <c r="H7" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F7</f>
-        <v>0.74</v>
-      </c>
-      <c r="I7" s="15">
-        <f t="shared" si="1"/>
+      <c r="I7" s="15" cm="1">
+        <f t="array" ref="I7">(H7+H6)/2*$E$3</f>
         <v>0.19749999999999998</v>
       </c>
-      <c r="J7" s="35">
-        <f t="shared" si="2"/>
-        <v>0.36499999999999999</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="20.399999999999999" customHeight="1">
+    </row>
+    <row r="8" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A8" s="28">
         <v>46225.385416666664</v>
       </c>
-      <c r="B8" s="37">
+      <c r="B8" s="38">
         <v>0.12</v>
       </c>
       <c r="C8" s="15" cm="1">
-        <f t="array" ref="C8">(B8+B7)/2*$D$3</f>
+        <f t="array" ref="C8">(B8+B7)/2*$E$3</f>
         <v>0.09</v>
       </c>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
-      <c r="G8" s="30">
-        <f t="shared" si="0"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="15" cm="1">
+        <f t="array" ref="H8">-B8+$F$3</f>
         <v>0.56999999999999995</v>
       </c>
-      <c r="H8" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F8</f>
-        <v>0.78</v>
-      </c>
-      <c r="I8" s="15">
-        <f t="shared" si="1"/>
+      <c r="I8" s="15" cm="1">
+        <f t="array" ref="I8">(H8+H7)/2*$E$3</f>
         <v>0.255</v>
       </c>
-      <c r="J8" s="35">
-        <f t="shared" si="2"/>
-        <v>0.38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="20.399999999999999" customHeight="1">
+    </row>
+    <row r="9" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A9" s="31">
         <v>46225.385416666664</v>
       </c>
-      <c r="B9" s="37">
+      <c r="B9" s="38">
         <v>0.71</v>
       </c>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
-      <c r="G9" s="30">
-        <f>$F$3-B9</f>
+      <c r="G9" s="16"/>
+      <c r="H9" s="15" cm="1">
+        <f t="array" ref="H9">-B9+$G$3</f>
         <v>0.59000000000000008</v>
       </c>
-      <c r="H9" s="11">
-        <v>0.78</v>
-      </c>
       <c r="I9" s="16"/>
     </row>
-    <row r="10" spans="1:10" ht="20.399999999999999" customHeight="1">
+    <row r="10" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A10" s="28">
         <v>46225.40625</v>
       </c>
-      <c r="B10" s="37">
+      <c r="B10" s="38">
         <v>0.64</v>
       </c>
       <c r="C10" s="15" cm="1">
-        <f t="array" ref="C10">(B10+B9)/2*$D$3</f>
+        <f t="array" ref="C10">(B10+B9)/2*$E$3</f>
         <v>0.33750000000000002</v>
       </c>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
-      <c r="G10" s="30">
-        <f t="shared" ref="G10:G24" si="3">$F$3-B10</f>
+      <c r="G10" s="16"/>
+      <c r="H10" s="15" cm="1">
+        <f t="array" ref="H10">-B10+$G$3</f>
         <v>0.66</v>
       </c>
-      <c r="H10" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F10</f>
-        <v>0.81</v>
-      </c>
-      <c r="I10" s="15">
-        <f>(G10+G9)/2*$D$3</f>
+      <c r="I10" s="15" cm="1">
+        <f t="array" ref="I10">(H10+H9)/2*$E$3</f>
         <v>0.3125</v>
       </c>
-      <c r="J10" s="35">
-        <f t="shared" si="2"/>
-        <v>0.39750000000000002</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="20.399999999999999" customHeight="1">
+    </row>
+    <row r="11" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A11" s="28">
         <v>46225.427083333336</v>
       </c>
-      <c r="B11" s="37">
+      <c r="B11" s="38">
         <v>0.54</v>
       </c>
       <c r="C11" s="15" cm="1">
-        <f t="array" ref="C11">(B11+B10)/2*$D$3</f>
+        <f t="array" ref="C11">(B11+B10)/2*$E$3</f>
         <v>0.29500000000000004</v>
       </c>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
-      <c r="G11" s="30">
-        <f t="shared" si="3"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="15" cm="1">
+        <f t="array" ref="H11">-B11+$G$3</f>
         <v>0.76</v>
       </c>
-      <c r="H11" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F11</f>
-        <v>0.84000000000000008</v>
-      </c>
-      <c r="I11" s="15">
-        <f t="shared" ref="I11:I24" si="4">(G11+G10)/2*$D$3</f>
+      <c r="I11" s="15" cm="1">
+        <f t="array" ref="I11">(H11+H10)/2*$E$3</f>
         <v>0.35499999999999998</v>
       </c>
-      <c r="J11" s="35">
-        <f t="shared" si="2"/>
-        <v>0.41250000000000003</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="20.399999999999999" customHeight="1">
+    </row>
+    <row r="12" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A12" s="28">
         <v>46225.447916666664</v>
       </c>
-      <c r="B12" s="37">
+      <c r="B12" s="38">
         <v>0.47</v>
       </c>
       <c r="C12" s="15" cm="1">
-        <f t="array" ref="C12">(B12+B11)/2*$D$3</f>
+        <f t="array" ref="C12">(B12+B11)/2*$E$3</f>
         <v>0.2525</v>
       </c>
       <c r="D12" s="16"/>
       <c r="E12" s="16"/>
       <c r="F12" s="16"/>
-      <c r="G12" s="30">
-        <f t="shared" si="3"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="15" cm="1">
+        <f t="array" ref="H12">-B12+$G$3</f>
         <v>0.83000000000000007</v>
       </c>
-      <c r="H12" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F12</f>
-        <v>0.87000000000000011</v>
-      </c>
-      <c r="I12" s="15">
-        <f t="shared" si="4"/>
+      <c r="I12" s="15" cm="1">
+        <f t="array" ref="I12">(H12+H11)/2*$E$3</f>
         <v>0.39750000000000002</v>
       </c>
-      <c r="J12" s="35">
-        <f t="shared" si="2"/>
-        <v>0.42750000000000005</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="20.399999999999999" customHeight="1">
+    </row>
+    <row r="13" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A13" s="28">
         <v>46225.46875</v>
       </c>
-      <c r="B13" s="37">
+      <c r="B13" s="38">
         <v>0.4</v>
       </c>
       <c r="C13" s="15" cm="1">
-        <f t="array" ref="C13">(B13+B12)/2*$D$3</f>
+        <f t="array" ref="C13">(B13+B12)/2*$E$3</f>
         <v>0.2175</v>
       </c>
       <c r="D13" s="16"/>
       <c r="E13" s="16"/>
       <c r="F13" s="16"/>
-      <c r="G13" s="30">
-        <f t="shared" si="3"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="15" cm="1">
+        <f t="array" ref="H13">-B13+$G$3</f>
         <v>0.9</v>
       </c>
-      <c r="H13" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F13</f>
-        <v>0.88000000000000012</v>
-      </c>
-      <c r="I13" s="15">
-        <f t="shared" si="4"/>
+      <c r="I13" s="15" cm="1">
+        <f t="array" ref="I13">(H13+H12)/2*$E$3</f>
         <v>0.4325</v>
       </c>
-      <c r="J13" s="35">
-        <f t="shared" si="2"/>
-        <v>0.43750000000000006</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="20.399999999999999" customHeight="1">
+    </row>
+    <row r="14" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A14" s="28">
         <v>46225.489583333336</v>
       </c>
-      <c r="B14" s="37">
+      <c r="B14" s="38">
         <v>0.36</v>
       </c>
       <c r="C14" s="15" cm="1">
-        <f t="array" ref="C14">(B14+B13)/2*$D$3</f>
+        <f t="array" ref="C14">(B14+B13)/2*$E$3</f>
         <v>0.19</v>
       </c>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
       <c r="F14" s="16"/>
-      <c r="G14" s="30">
-        <f t="shared" si="3"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="15" cm="1">
+        <f t="array" ref="H14">-B14+$G$3</f>
         <v>0.94000000000000006</v>
       </c>
-      <c r="H14" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F14</f>
-        <v>0.9</v>
-      </c>
-      <c r="I14" s="15">
-        <f t="shared" si="4"/>
+      <c r="I14" s="15" cm="1">
+        <f t="array" ref="I14">(H14+H13)/2*$E$3</f>
         <v>0.46</v>
       </c>
-      <c r="J14" s="35">
-        <f t="shared" si="2"/>
-        <v>0.44500000000000006</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="20.399999999999999" customHeight="1">
+    </row>
+    <row r="15" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A15" s="28">
         <v>46225.510416666664</v>
       </c>
-      <c r="B15" s="37">
+      <c r="B15" s="38">
         <v>0.34</v>
       </c>
       <c r="C15" s="15" cm="1">
-        <f t="array" ref="C15">(B15+B14)/2*$D$3</f>
+        <f t="array" ref="C15">(B15+B14)/2*$E$3</f>
         <v>0.17499999999999999</v>
       </c>
       <c r="D15" s="16"/>
       <c r="E15" s="16"/>
       <c r="F15" s="16"/>
-      <c r="G15" s="30">
-        <f t="shared" si="3"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="15" cm="1">
+        <f t="array" ref="H15">-B15+$G$3</f>
         <v>0.96</v>
       </c>
-      <c r="H15" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F15</f>
-        <v>0.9</v>
-      </c>
-      <c r="I15" s="15">
-        <f t="shared" si="4"/>
+      <c r="I15" s="15" cm="1">
+        <f t="array" ref="I15">(H15+H14)/2*$E$3</f>
         <v>0.47499999999999998</v>
       </c>
-      <c r="J15" s="35">
-        <f t="shared" si="2"/>
-        <v>0.45</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="20.399999999999999" customHeight="1">
+    </row>
+    <row r="16" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A16" s="28">
         <v>46225.53125</v>
       </c>
-      <c r="B16" s="37">
+      <c r="B16" s="38">
         <v>0.32</v>
       </c>
       <c r="C16" s="15" cm="1">
-        <f t="array" ref="C16">(B16+B15)/2*$D$3</f>
+        <f t="array" ref="C16">(B16+B15)/2*$E$3</f>
         <v>0.16500000000000001</v>
       </c>
       <c r="D16" s="16"/>
       <c r="E16" s="16"/>
       <c r="F16" s="16"/>
-      <c r="G16" s="30">
-        <f t="shared" si="3"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="15" cm="1">
+        <f t="array" ref="H16">-B16+$G$3</f>
         <v>0.98</v>
       </c>
-      <c r="H16" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F16</f>
-        <v>0.91</v>
-      </c>
-      <c r="I16" s="15">
-        <f t="shared" si="4"/>
+      <c r="I16" s="15" cm="1">
+        <f t="array" ref="I16">(H16+H15)/2*$E$3</f>
         <v>0.48499999999999999</v>
       </c>
-      <c r="J16" s="35">
-        <f t="shared" si="2"/>
-        <v>0.45250000000000001</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="20.399999999999999" customHeight="1">
+    </row>
+    <row r="17" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A17" s="28">
         <v>46225.552083333336</v>
       </c>
-      <c r="B17" s="37">
+      <c r="B17" s="38">
         <v>0.33</v>
       </c>
       <c r="C17" s="15" cm="1">
-        <f t="array" ref="C17">(B17+B16)/2*$D$3</f>
+        <f t="array" ref="C17">(B17+B16)/2*$E$3</f>
         <v>0.16250000000000001</v>
       </c>
       <c r="D17" s="16"/>
       <c r="E17" s="16"/>
       <c r="F17" s="16"/>
-      <c r="G17" s="30">
-        <f t="shared" si="3"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="15" cm="1">
+        <f t="array" ref="H17">-B17+$G$3</f>
         <v>0.97</v>
       </c>
-      <c r="H17" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F17</f>
-        <v>0.91</v>
-      </c>
-      <c r="I17" s="15">
-        <f t="shared" si="4"/>
+      <c r="I17" s="15" cm="1">
+        <f t="array" ref="I17">(H17+H16)/2*$E$3</f>
         <v>0.48749999999999999</v>
       </c>
-      <c r="J17" s="35">
-        <f t="shared" si="2"/>
-        <v>0.45500000000000002</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="20.399999999999999" customHeight="1">
+    </row>
+    <row r="18" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A18" s="28">
         <v>46225.572916666664</v>
       </c>
-      <c r="B18" s="37">
+      <c r="B18" s="38">
         <v>0.34</v>
       </c>
       <c r="C18" s="15" cm="1">
-        <f t="array" ref="C18">(B18+B17)/2*$D$3</f>
+        <f t="array" ref="C18">(B18+B17)/2*$E$3</f>
         <v>0.16750000000000001</v>
       </c>
       <c r="D18" s="16"/>
       <c r="E18" s="16"/>
       <c r="F18" s="16"/>
-      <c r="G18" s="30">
-        <f t="shared" si="3"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="15" cm="1">
+        <f t="array" ref="H18">-B18+$G$3</f>
         <v>0.96</v>
       </c>
-      <c r="H18" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F18</f>
-        <v>0.9</v>
-      </c>
-      <c r="I18" s="15">
-        <f t="shared" si="4"/>
+      <c r="I18" s="15" cm="1">
+        <f t="array" ref="I18">(H18+H17)/2*$E$3</f>
         <v>0.48249999999999998</v>
       </c>
-      <c r="J18" s="35">
-        <f t="shared" si="2"/>
-        <v>0.45250000000000001</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="20.399999999999999" customHeight="1">
+    </row>
+    <row r="19" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A19" s="28">
         <v>46225.59375</v>
       </c>
-      <c r="B19" s="37">
+      <c r="B19" s="38">
         <v>0.38</v>
       </c>
       <c r="C19" s="15" cm="1">
-        <f t="array" ref="C19">(B19+B18)/2*$D$3</f>
+        <f t="array" ref="C19">(B19+B18)/2*$E$3</f>
         <v>0.18</v>
       </c>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
-      <c r="G19" s="30">
-        <f t="shared" si="3"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="15" cm="1">
+        <f t="array" ref="H19">-B19+$G$3</f>
         <v>0.92</v>
       </c>
-      <c r="H19" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F19</f>
-        <v>0.9</v>
-      </c>
-      <c r="I19" s="15">
-        <f t="shared" si="4"/>
+      <c r="I19" s="15" cm="1">
+        <f t="array" ref="I19">(H19+H18)/2*$E$3</f>
         <v>0.47</v>
       </c>
-      <c r="J19" s="35">
-        <f t="shared" si="2"/>
-        <v>0.45</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="20.399999999999999" customHeight="1">
+    </row>
+    <row r="20" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A20" s="28">
         <v>46225.614583333336</v>
       </c>
-      <c r="B20" s="37">
+      <c r="B20" s="38">
         <v>0.42</v>
       </c>
       <c r="C20" s="15" cm="1">
-        <f t="array" ref="C20">(B20+B19)/2*$D$3</f>
+        <f t="array" ref="C20">(B20+B19)/2*$E$3</f>
         <v>0.2</v>
       </c>
       <c r="D20" s="16"/>
       <c r="E20" s="16"/>
       <c r="F20" s="16"/>
-      <c r="G20" s="30">
-        <f t="shared" si="3"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="15" cm="1">
+        <f t="array" ref="H20">-B20+$G$3</f>
         <v>0.88000000000000012</v>
       </c>
-      <c r="H20" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F20</f>
-        <v>0.88000000000000012</v>
-      </c>
-      <c r="I20" s="15">
-        <f t="shared" si="4"/>
+      <c r="I20" s="15" cm="1">
+        <f t="array" ref="I20">(H20+H19)/2*$E$3</f>
         <v>0.45000000000000007</v>
       </c>
-      <c r="J20" s="35">
-        <f t="shared" si="2"/>
-        <v>0.44500000000000006</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="20.399999999999999" customHeight="1">
+    </row>
+    <row r="21" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A21" s="28">
         <v>46225.635416666664</v>
       </c>
-      <c r="B21" s="37">
+      <c r="B21" s="38">
         <v>0.47</v>
       </c>
       <c r="C21" s="15" cm="1">
-        <f t="array" ref="C21">(B21+B20)/2*$D$3</f>
+        <f t="array" ref="C21">(B21+B20)/2*$E$3</f>
         <v>0.22249999999999998</v>
       </c>
       <c r="D21" s="16"/>
       <c r="E21" s="16"/>
       <c r="F21" s="16"/>
-      <c r="G21" s="30">
-        <f t="shared" si="3"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="15" cm="1">
+        <f t="array" ref="H21">-B21+$G$3</f>
         <v>0.83000000000000007</v>
       </c>
-      <c r="H21" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F21</f>
-        <v>0.8600000000000001</v>
-      </c>
-      <c r="I21" s="15">
-        <f t="shared" si="4"/>
+      <c r="I21" s="15" cm="1">
+        <f t="array" ref="I21">(H21+H20)/2*$E$3</f>
         <v>0.42750000000000005</v>
       </c>
-      <c r="J21" s="35">
-        <f t="shared" si="2"/>
-        <v>0.43500000000000005</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="20.399999999999999" customHeight="1">
+    </row>
+    <row r="22" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A22" s="28">
         <v>46225.65625</v>
       </c>
-      <c r="B22" s="37">
+      <c r="B22" s="38">
         <v>0.55000000000000004</v>
       </c>
       <c r="C22" s="15" cm="1">
-        <f t="array" ref="C22">(B22+B21)/2*$D$3</f>
+        <f t="array" ref="C22">(B22+B21)/2*$E$3</f>
         <v>0.255</v>
       </c>
       <c r="D22" s="16"/>
       <c r="E22" s="16"/>
       <c r="F22" s="16"/>
-      <c r="G22" s="30">
-        <f t="shared" si="3"/>
+      <c r="G22" s="16"/>
+      <c r="H22" s="15" cm="1">
+        <f t="array" ref="H22">-B22+$G$3</f>
         <v>0.75</v>
       </c>
-      <c r="H22" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F22</f>
-        <v>0.84000000000000008</v>
-      </c>
-      <c r="I22" s="15">
-        <f t="shared" si="4"/>
+      <c r="I22" s="15" cm="1">
+        <f t="array" ref="I22">(H22+H21)/2*$E$3</f>
         <v>0.39500000000000002</v>
       </c>
-      <c r="J22" s="35">
-        <f t="shared" si="2"/>
-        <v>0.42500000000000004</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="20.399999999999999" customHeight="1">
+    </row>
+    <row r="23" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A23" s="28">
         <v>46225.677083333336</v>
       </c>
-      <c r="B23" s="37">
+      <c r="B23" s="38">
         <v>0.65</v>
       </c>
       <c r="C23" s="15" cm="1">
-        <f t="array" ref="C23">(B23+B22)/2*$D$3</f>
+        <f t="array" ref="C23">(B23+B22)/2*$E$3</f>
         <v>0.30000000000000004</v>
       </c>
       <c r="D23" s="16"/>
       <c r="E23" s="16"/>
       <c r="F23" s="16"/>
-      <c r="G23" s="30">
-        <f t="shared" si="3"/>
+      <c r="G23" s="16"/>
+      <c r="H23" s="15" cm="1">
+        <f t="array" ref="H23">-B23+$G$3</f>
         <v>0.65</v>
       </c>
-      <c r="H23" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F23</f>
-        <v>0.82000000000000006</v>
-      </c>
-      <c r="I23" s="15">
-        <f t="shared" si="4"/>
+      <c r="I23" s="15" cm="1">
+        <f t="array" ref="I23">(H23+H22)/2*$E$3</f>
         <v>0.35</v>
       </c>
-      <c r="J23" s="35">
-        <f t="shared" si="2"/>
-        <v>0.41500000000000004</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="20.399999999999999" customHeight="1">
+    </row>
+    <row r="24" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A24" s="28">
         <v>46225.697916666664</v>
       </c>
-      <c r="B24" s="37">
+      <c r="B24" s="38">
         <v>0.75</v>
       </c>
       <c r="C24" s="15" cm="1">
-        <f t="array" ref="C24">(B24+B23)/2*$D$3</f>
+        <f t="array" ref="C24">(B24+B23)/2*$E$3</f>
         <v>0.35</v>
       </c>
       <c r="D24" s="16"/>
       <c r="E24" s="16"/>
       <c r="F24" s="16"/>
-      <c r="G24" s="30">
-        <f t="shared" si="3"/>
+      <c r="G24" s="16"/>
+      <c r="H24" s="15" cm="1">
+        <f t="array" ref="H24">-B24+$G$3</f>
         <v>0.55000000000000004</v>
       </c>
-      <c r="H24" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F24</f>
-        <v>0.78</v>
-      </c>
-      <c r="I24" s="15">
-        <f t="shared" si="4"/>
+      <c r="I24" s="15" cm="1">
+        <f t="array" ref="I24">(H24+H23)/2*$E$3</f>
         <v>0.30000000000000004</v>
       </c>
-      <c r="J24" s="35">
-        <f t="shared" si="2"/>
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="20.399999999999999" customHeight="1">
+    </row>
+    <row r="25" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A25" s="28">
         <v>46225.697916666664</v>
       </c>
-      <c r="B25" s="37">
+      <c r="B25" s="38">
         <v>0.1</v>
       </c>
       <c r="C25" s="16"/>
       <c r="D25" s="16"/>
       <c r="E25" s="16"/>
       <c r="F25" s="16"/>
-      <c r="G25" s="30">
-        <f>$E$3-B25</f>
+      <c r="G25" s="16"/>
+      <c r="H25" s="15" cm="1">
+        <f t="array" ref="H25">-B25+$F$3</f>
         <v>0.59</v>
       </c>
-      <c r="H25" s="11">
-        <v>0.78</v>
-      </c>
       <c r="I25" s="16"/>
     </row>
-    <row r="26" spans="1:10" ht="20.399999999999999" customHeight="1">
+    <row r="26" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A26" s="28">
         <v>46225.71875</v>
       </c>
-      <c r="B26" s="37">
+      <c r="B26" s="38">
         <v>0.2</v>
       </c>
       <c r="C26" s="15" cm="1">
-        <f t="array" ref="C26">(B26+B25)/2*$D$3</f>
+        <f t="array" ref="C26">(B26+B25)/2*$E$3</f>
         <v>7.5000000000000011E-2</v>
       </c>
       <c r="D26" s="16"/>
       <c r="E26" s="16"/>
       <c r="F26" s="16"/>
-      <c r="G26" s="30">
-        <f>$E$3-B26</f>
+      <c r="G26" s="16"/>
+      <c r="H26" s="15" cm="1">
+        <f t="array" ref="H26">-B26+$F$3</f>
         <v>0.48999999999999994</v>
       </c>
-      <c r="H26" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F26</f>
-        <v>0.74</v>
-      </c>
-      <c r="I26" s="15">
-        <f>(G26+G25)/2*$D$3</f>
+      <c r="I26" s="15" cm="1">
+        <f t="array" ref="I26">(H26+H25)/2*$E$3</f>
         <v>0.26999999999999996</v>
       </c>
-      <c r="J26" s="35">
-        <f t="shared" si="2"/>
-        <v>0.38</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="20.399999999999999" customHeight="1">
+    </row>
+    <row r="27" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A27" s="28">
         <v>46225.739583333336</v>
       </c>
-      <c r="B27" s="37">
+      <c r="B27" s="38">
         <v>0.32</v>
       </c>
       <c r="C27" s="15" cm="1">
-        <f t="array" ref="C27">(B27+B26)/2*$D$3</f>
+        <f t="array" ref="C27">(B27+B26)/2*$E$3</f>
         <v>0.13</v>
       </c>
       <c r="D27" s="16"/>
       <c r="E27" s="16"/>
       <c r="F27" s="16"/>
-      <c r="G27" s="30">
-        <f>$E$3-B27</f>
+      <c r="G27" s="16"/>
+      <c r="H27" s="15" cm="1">
+        <f t="array" ref="H27">-B27+$F$3</f>
         <v>0.36999999999999994</v>
       </c>
-      <c r="H27" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F27</f>
-        <v>0.75</v>
-      </c>
-      <c r="I27" s="15">
-        <f t="shared" ref="I27:I30" si="5">(G27+G26)/2*$D$3</f>
+      <c r="I27" s="15" cm="1">
+        <f t="array" ref="I27">(H27+H26)/2*$E$3</f>
         <v>0.21499999999999997</v>
       </c>
-      <c r="J27" s="35">
-        <f t="shared" si="2"/>
-        <v>0.3725</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="20.399999999999999" customHeight="1">
+    </row>
+    <row r="28" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A28" s="28">
         <v>46225.760416666664</v>
       </c>
-      <c r="B28" s="37">
+      <c r="B28" s="38">
         <v>0.45</v>
       </c>
       <c r="C28" s="15" cm="1">
-        <f t="array" ref="C28">(B28+B27)/2*$D$3</f>
+        <f t="array" ref="C28">(B28+B27)/2*$E$3</f>
         <v>0.1925</v>
       </c>
       <c r="D28" s="16"/>
       <c r="E28" s="16"/>
       <c r="F28" s="16"/>
-      <c r="G28" s="30">
-        <f>$E$3-B28</f>
+      <c r="G28" s="16"/>
+      <c r="H28" s="15" cm="1">
+        <f t="array" ref="H28">-B28+$F$3</f>
         <v>0.23999999999999994</v>
       </c>
-      <c r="H28" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F28</f>
-        <v>0.65999999999999992</v>
-      </c>
-      <c r="I28" s="15">
-        <f t="shared" si="5"/>
+      <c r="I28" s="15" cm="1">
+        <f t="array" ref="I28">(H28+H27)/2*$E$3</f>
         <v>0.15249999999999997</v>
       </c>
-      <c r="J28" s="35">
-        <f t="shared" si="2"/>
-        <v>0.35249999999999998</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="20.399999999999999" customHeight="1">
+    </row>
+    <row r="29" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A29" s="28">
         <v>0.78125</v>
       </c>
-      <c r="B29" s="37">
-        <v>0.59</v>
-      </c>
+      <c r="B29" s="38"/>
       <c r="C29" s="15"/>
       <c r="D29" s="16"/>
       <c r="E29" s="16"/>
       <c r="F29" s="16"/>
-      <c r="G29" s="30">
-        <f>$E$3-B29</f>
-        <v>9.9999999999999978E-2</v>
-      </c>
-      <c r="H29" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F29</f>
-        <v>0.49999999999999994</v>
-      </c>
-      <c r="I29" s="15">
-        <f t="shared" si="5"/>
-        <v>8.4999999999999978E-2</v>
-      </c>
-      <c r="J29" s="35">
-        <f t="shared" si="2"/>
-        <v>0.28999999999999998</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" ht="20.399999999999999" customHeight="1">
+      <c r="G29" s="16"/>
+      <c r="H29" s="15"/>
+      <c r="I29" s="15"/>
+    </row>
+    <row r="30" spans="1:9" ht="20.399999999999999" customHeight="1">
       <c r="A30" s="28">
         <v>0.80208333333333337</v>
       </c>
-      <c r="B30" s="37">
-        <v>0.72</v>
-      </c>
+      <c r="B30" s="38"/>
       <c r="C30" s="15"/>
       <c r="D30" s="16"/>
       <c r="E30" s="16"/>
       <c r="F30" s="16"/>
-      <c r="G30" s="30">
-        <v>0</v>
-      </c>
-      <c r="H30" s="11">
-        <f>'Solar Panel Comparisons - Solar'!F30</f>
-        <v>0.28999999999999992</v>
-      </c>
-      <c r="I30" s="15">
-        <f t="shared" si="5"/>
-        <v>2.4999999999999994E-2</v>
-      </c>
-      <c r="J30" s="35">
-        <f t="shared" si="2"/>
-        <v>0.19749999999999995</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" ht="20.399999999999999" customHeight="1">
-      <c r="A31" s="33" t="s">
-        <v>37</v>
-      </c>
+      <c r="G30" s="16"/>
+      <c r="H30" s="15"/>
+      <c r="I30" s="15"/>
+    </row>
+    <row r="31" spans="1:9" ht="20.399999999999999" customHeight="1">
+      <c r="A31" s="33"/>
       <c r="B31" s="33"/>
       <c r="C31" s="15" cm="1">
         <f t="array" ref="C31">SUM(C3:C28)</f>
@@ -17518,12 +17992,8 @@
         <f t="array" ref="I31">SUM(I3:I28)</f>
         <v>7.6149999999999993</v>
       </c>
-      <c r="J31" s="35">
-        <f>SUM(J4:J30)</f>
-        <v>9.65</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" ht="19.95" customHeight="1">
+    </row>
+    <row r="32" spans="1:9" ht="19.95" customHeight="1">
       <c r="A32" s="33"/>
     </row>
     <row r="33" spans="1:1" ht="19.95" customHeight="1">
@@ -17542,4 +18012,836 @@
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E54"/>
+  <sheetFormatPr defaultRowHeight="13.2"/>
+  <cols>
+    <col min="1" max="1" width="14.77734375" style="42" customWidth="1"/>
+    <col min="2" max="2" width="13" style="42" customWidth="1"/>
+    <col min="3" max="3" width="11.109375" style="42" customWidth="1"/>
+    <col min="4" max="4" width="9.109375" style="42"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="24.6">
+      <c r="A1" s="44" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="42" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" s="40" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" s="40" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="41">
+        <v>46225.28125</v>
+      </c>
+      <c r="B2" s="42">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="C2" s="40">
+        <v>0.23</v>
+      </c>
+      <c r="D2" s="45">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="43">
+        <v>46225.302083333336</v>
+      </c>
+      <c r="B3" s="42">
+        <v>0.03</v>
+      </c>
+      <c r="C3" s="42">
+        <v>0.5</v>
+      </c>
+      <c r="D3" s="45">
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="43">
+        <v>46225.322916666664</v>
+      </c>
+      <c r="B4" s="42">
+        <v>0.13</v>
+      </c>
+      <c r="C4" s="42">
+        <v>0.67</v>
+      </c>
+      <c r="D4" s="45">
+        <v>0.74</v>
+      </c>
+      <c r="E4">
+        <v>0.53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="43">
+        <v>46225.34375</v>
+      </c>
+      <c r="B5" s="42">
+        <v>0.23</v>
+      </c>
+      <c r="C5" s="42">
+        <v>0.77</v>
+      </c>
+      <c r="D5" s="45">
+        <v>0.84</v>
+      </c>
+      <c r="E5">
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="43">
+        <v>46225.364583333336</v>
+      </c>
+      <c r="B6" s="42">
+        <v>0.37</v>
+      </c>
+      <c r="C6" s="42">
+        <v>0.85</v>
+      </c>
+      <c r="D6" s="45">
+        <v>0.86</v>
+      </c>
+      <c r="E6">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="43">
+        <v>46225.385416666664</v>
+      </c>
+      <c r="B7" s="42">
+        <v>0.49</v>
+      </c>
+      <c r="C7" s="42">
+        <v>0.89</v>
+      </c>
+      <c r="D7" s="42">
+        <v>0.9</v>
+      </c>
+      <c r="E7">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="43">
+        <v>46225.40625</v>
+      </c>
+      <c r="B8" s="42">
+        <v>0.6</v>
+      </c>
+      <c r="C8" s="42">
+        <v>0.94</v>
+      </c>
+      <c r="D8" s="42">
+        <v>0.93</v>
+      </c>
+      <c r="E8">
+        <v>0.87</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="43">
+        <v>46225.427083333336</v>
+      </c>
+      <c r="B9" s="42">
+        <v>0.7</v>
+      </c>
+      <c r="C9" s="42">
+        <v>0.96</v>
+      </c>
+      <c r="D9" s="42">
+        <v>0.96</v>
+      </c>
+      <c r="E9">
+        <v>0.92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="43">
+        <v>46225.447916666664</v>
+      </c>
+      <c r="B10" s="42">
+        <v>0.8</v>
+      </c>
+      <c r="C10" s="42">
+        <v>0.98</v>
+      </c>
+      <c r="D10" s="42">
+        <v>0.99</v>
+      </c>
+      <c r="E10">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="43">
+        <v>46225.46875</v>
+      </c>
+      <c r="B11" s="42">
+        <v>0.87</v>
+      </c>
+      <c r="C11" s="42">
+        <v>1</v>
+      </c>
+      <c r="D11" s="42">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>0.97</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="43">
+        <v>46225.489583333336</v>
+      </c>
+      <c r="B12" s="42">
+        <v>0.93</v>
+      </c>
+      <c r="C12" s="42">
+        <v>1</v>
+      </c>
+      <c r="D12" s="42">
+        <v>1.02</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="43">
+        <v>46225.510416666664</v>
+      </c>
+      <c r="B13" s="42">
+        <v>0.98</v>
+      </c>
+      <c r="C13" s="42">
+        <v>0.99</v>
+      </c>
+      <c r="D13" s="42">
+        <v>1.03</v>
+      </c>
+      <c r="E13">
+        <v>1.02</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="43">
+        <v>46225.53125</v>
+      </c>
+      <c r="B14" s="42">
+        <v>0.99</v>
+      </c>
+      <c r="C14" s="42">
+        <v>0.98</v>
+      </c>
+      <c r="D14" s="42">
+        <v>1.03</v>
+      </c>
+      <c r="E14">
+        <v>1.01</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="43">
+        <v>46225.552083333336</v>
+      </c>
+      <c r="B15" s="42">
+        <v>0.99</v>
+      </c>
+      <c r="C15" s="42">
+        <v>0.99</v>
+      </c>
+      <c r="D15" s="42">
+        <v>1.03</v>
+      </c>
+      <c r="E15">
+        <v>1.02</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="43">
+        <v>46225.572916666664</v>
+      </c>
+      <c r="B16" s="42">
+        <v>0.97</v>
+      </c>
+      <c r="C16" s="42">
+        <v>0.99</v>
+      </c>
+      <c r="D16" s="42">
+        <v>1.02</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="43">
+        <v>46225.59375</v>
+      </c>
+      <c r="B17" s="42">
+        <v>0.93</v>
+      </c>
+      <c r="C17" s="42">
+        <v>1</v>
+      </c>
+      <c r="D17" s="42">
+        <v>1.01</v>
+      </c>
+      <c r="E17">
+        <v>0.99</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="43">
+        <v>46225.614583333336</v>
+      </c>
+      <c r="B18" s="42">
+        <v>0.88</v>
+      </c>
+      <c r="C18" s="42">
+        <v>0.99</v>
+      </c>
+      <c r="D18" s="42">
+        <v>0.97</v>
+      </c>
+      <c r="E18">
+        <v>0.97</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="43">
+        <v>46225.635416666664</v>
+      </c>
+      <c r="B19" s="42">
+        <v>0.83</v>
+      </c>
+      <c r="C19" s="42">
+        <v>0.98</v>
+      </c>
+      <c r="D19" s="42">
+        <v>0.97</v>
+      </c>
+      <c r="E19">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="43">
+        <v>46225.65625</v>
+      </c>
+      <c r="B20" s="42">
+        <v>0.75</v>
+      </c>
+      <c r="C20" s="42">
+        <v>0.95</v>
+      </c>
+      <c r="D20" s="42">
+        <v>0.95</v>
+      </c>
+      <c r="E20">
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" s="43">
+        <v>46225.677083333336</v>
+      </c>
+      <c r="B21" s="42">
+        <v>0.64</v>
+      </c>
+      <c r="C21" s="42">
+        <v>0.93</v>
+      </c>
+      <c r="D21" s="42">
+        <v>0.92</v>
+      </c>
+      <c r="E21">
+        <v>0.89</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" s="43">
+        <v>46225.697916666664</v>
+      </c>
+      <c r="B22" s="42">
+        <v>0.53</v>
+      </c>
+      <c r="C22" s="42">
+        <v>0.89</v>
+      </c>
+      <c r="D22" s="42">
+        <v>0.88</v>
+      </c>
+      <c r="E22">
+        <v>0.89</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" s="43">
+        <v>46225.71875</v>
+      </c>
+      <c r="B23" s="42">
+        <v>0.36</v>
+      </c>
+      <c r="C23" s="42">
+        <v>0.89</v>
+      </c>
+      <c r="D23" s="42">
+        <v>0.86</v>
+      </c>
+      <c r="E23">
+        <v>0.83</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" s="43">
+        <v>46225.739583333336</v>
+      </c>
+      <c r="B24" s="42">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="C24" s="42">
+        <v>0.84</v>
+      </c>
+      <c r="D24" s="42">
+        <v>0.87</v>
+      </c>
+      <c r="E24">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" s="43">
+        <v>46225.760416666664</v>
+      </c>
+      <c r="B25" s="42">
+        <v>0.16</v>
+      </c>
+      <c r="C25" s="42">
+        <v>0.74</v>
+      </c>
+      <c r="D25" s="42">
+        <v>0.78</v>
+      </c>
+      <c r="E25">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" s="43">
+        <v>0.78125</v>
+      </c>
+      <c r="B26" s="40">
+        <v>0.05</v>
+      </c>
+      <c r="C26" s="42">
+        <v>0.6</v>
+      </c>
+      <c r="D26" s="42">
+        <v>0.62</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" s="43">
+        <v>0.80208333333333337</v>
+      </c>
+      <c r="B27" s="42">
+        <v>0.01</v>
+      </c>
+      <c r="C27" s="42">
+        <v>0.3</v>
+      </c>
+      <c r="D27" s="42">
+        <v>0.41</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="B29" s="42">
+        <f>(B3+B2)/2*0.5</f>
+        <v>8.7499999999999991E-3</v>
+      </c>
+      <c r="C29" s="42">
+        <f>(C3+C2)/2*0.5</f>
+        <v>0.1825</v>
+      </c>
+      <c r="D29" s="42">
+        <f>(D3+D2)/2*0.5</f>
+        <v>0.22500000000000001</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="B30" s="42">
+        <f t="shared" ref="B30:D53" si="0">(B4+B3)/2*0.5</f>
+        <v>0.04</v>
+      </c>
+      <c r="C30" s="42">
+        <f t="shared" si="0"/>
+        <v>0.29249999999999998</v>
+      </c>
+      <c r="D30" s="42">
+        <f t="shared" si="0"/>
+        <v>0.32250000000000001</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="B31" s="42">
+        <f t="shared" si="0"/>
+        <v>0.09</v>
+      </c>
+      <c r="C31" s="42">
+        <f t="shared" si="0"/>
+        <v>0.36</v>
+      </c>
+      <c r="D31" s="42">
+        <f t="shared" si="0"/>
+        <v>0.39500000000000002</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="B32" s="42">
+        <f t="shared" si="0"/>
+        <v>0.15</v>
+      </c>
+      <c r="C32" s="42">
+        <f t="shared" si="0"/>
+        <v>0.40500000000000003</v>
+      </c>
+      <c r="D32" s="42">
+        <f t="shared" si="0"/>
+        <v>0.42499999999999999</v>
+      </c>
+    </row>
+    <row r="33" spans="2:4">
+      <c r="B33" s="42">
+        <f t="shared" si="0"/>
+        <v>0.215</v>
+      </c>
+      <c r="C33" s="42">
+        <f t="shared" si="0"/>
+        <v>0.435</v>
+      </c>
+      <c r="D33" s="42">
+        <f t="shared" si="0"/>
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="34" spans="2:4">
+      <c r="B34" s="42">
+        <f t="shared" si="0"/>
+        <v>0.27249999999999996</v>
+      </c>
+      <c r="C34" s="42">
+        <f t="shared" si="0"/>
+        <v>0.45750000000000002</v>
+      </c>
+      <c r="D34" s="42">
+        <f t="shared" si="0"/>
+        <v>0.45750000000000002</v>
+      </c>
+    </row>
+    <row r="35" spans="2:4">
+      <c r="B35" s="42">
+        <f t="shared" si="0"/>
+        <v>0.32499999999999996</v>
+      </c>
+      <c r="C35" s="42">
+        <f t="shared" si="0"/>
+        <v>0.47499999999999998</v>
+      </c>
+      <c r="D35" s="42">
+        <f t="shared" si="0"/>
+        <v>0.47250000000000003</v>
+      </c>
+    </row>
+    <row r="36" spans="2:4">
+      <c r="B36" s="42">
+        <f t="shared" si="0"/>
+        <v>0.375</v>
+      </c>
+      <c r="C36" s="42">
+        <f t="shared" si="0"/>
+        <v>0.48499999999999999</v>
+      </c>
+      <c r="D36" s="42">
+        <f t="shared" si="0"/>
+        <v>0.48749999999999999</v>
+      </c>
+    </row>
+    <row r="37" spans="2:4">
+      <c r="B37" s="42">
+        <f t="shared" si="0"/>
+        <v>0.41749999999999998</v>
+      </c>
+      <c r="C37" s="42">
+        <f t="shared" si="0"/>
+        <v>0.495</v>
+      </c>
+      <c r="D37" s="42">
+        <f t="shared" si="0"/>
+        <v>0.4975</v>
+      </c>
+    </row>
+    <row r="38" spans="2:4">
+      <c r="B38" s="42">
+        <f t="shared" si="0"/>
+        <v>0.45</v>
+      </c>
+      <c r="C38" s="42">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+      <c r="D38" s="42">
+        <f t="shared" si="0"/>
+        <v>0.505</v>
+      </c>
+    </row>
+    <row r="39" spans="2:4">
+      <c r="B39" s="42">
+        <f t="shared" si="0"/>
+        <v>0.47750000000000004</v>
+      </c>
+      <c r="C39" s="42">
+        <f t="shared" si="0"/>
+        <v>0.4975</v>
+      </c>
+      <c r="D39" s="42">
+        <f t="shared" si="0"/>
+        <v>0.51249999999999996</v>
+      </c>
+    </row>
+    <row r="40" spans="2:4">
+      <c r="B40" s="42">
+        <f t="shared" si="0"/>
+        <v>0.49249999999999999</v>
+      </c>
+      <c r="C40" s="42">
+        <f t="shared" si="0"/>
+        <v>0.49249999999999999</v>
+      </c>
+      <c r="D40" s="42">
+        <f t="shared" si="0"/>
+        <v>0.51500000000000001</v>
+      </c>
+    </row>
+    <row r="41" spans="2:4">
+      <c r="B41" s="42">
+        <f t="shared" si="0"/>
+        <v>0.495</v>
+      </c>
+      <c r="C41" s="42">
+        <f t="shared" si="0"/>
+        <v>0.49249999999999999</v>
+      </c>
+      <c r="D41" s="42">
+        <f t="shared" si="0"/>
+        <v>0.51500000000000001</v>
+      </c>
+    </row>
+    <row r="42" spans="2:4">
+      <c r="B42" s="42">
+        <f t="shared" si="0"/>
+        <v>0.49</v>
+      </c>
+      <c r="C42" s="42">
+        <f t="shared" si="0"/>
+        <v>0.495</v>
+      </c>
+      <c r="D42" s="42">
+        <f t="shared" si="0"/>
+        <v>0.51249999999999996</v>
+      </c>
+    </row>
+    <row r="43" spans="2:4">
+      <c r="B43" s="42">
+        <f t="shared" si="0"/>
+        <v>0.47499999999999998</v>
+      </c>
+      <c r="C43" s="42">
+        <f t="shared" si="0"/>
+        <v>0.4975</v>
+      </c>
+      <c r="D43" s="42">
+        <f t="shared" si="0"/>
+        <v>0.50750000000000006</v>
+      </c>
+    </row>
+    <row r="44" spans="2:4">
+      <c r="B44" s="42">
+        <f t="shared" si="0"/>
+        <v>0.45250000000000001</v>
+      </c>
+      <c r="C44" s="42">
+        <f t="shared" si="0"/>
+        <v>0.4975</v>
+      </c>
+      <c r="D44" s="42">
+        <f t="shared" si="0"/>
+        <v>0.495</v>
+      </c>
+    </row>
+    <row r="45" spans="2:4">
+      <c r="B45" s="42">
+        <f t="shared" si="0"/>
+        <v>0.42749999999999999</v>
+      </c>
+      <c r="C45" s="42">
+        <f t="shared" si="0"/>
+        <v>0.49249999999999999</v>
+      </c>
+      <c r="D45" s="42">
+        <f t="shared" si="0"/>
+        <v>0.48499999999999999</v>
+      </c>
+    </row>
+    <row r="46" spans="2:4">
+      <c r="B46" s="42">
+        <f t="shared" si="0"/>
+        <v>0.39500000000000002</v>
+      </c>
+      <c r="C46" s="42">
+        <f t="shared" si="0"/>
+        <v>0.48249999999999998</v>
+      </c>
+      <c r="D46" s="42">
+        <f t="shared" si="0"/>
+        <v>0.48</v>
+      </c>
+    </row>
+    <row r="47" spans="2:4">
+      <c r="B47" s="42">
+        <f t="shared" si="0"/>
+        <v>0.34750000000000003</v>
+      </c>
+      <c r="C47" s="42">
+        <f t="shared" si="0"/>
+        <v>0.47</v>
+      </c>
+      <c r="D47" s="42">
+        <f t="shared" si="0"/>
+        <v>0.46750000000000003</v>
+      </c>
+    </row>
+    <row r="48" spans="2:4">
+      <c r="B48" s="42">
+        <f t="shared" si="0"/>
+        <v>0.29249999999999998</v>
+      </c>
+      <c r="C48" s="42">
+        <f t="shared" si="0"/>
+        <v>0.45500000000000002</v>
+      </c>
+      <c r="D48" s="42">
+        <f t="shared" si="0"/>
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
+      <c r="B49" s="42">
+        <f t="shared" si="0"/>
+        <v>0.2225</v>
+      </c>
+      <c r="C49" s="42">
+        <f t="shared" si="0"/>
+        <v>0.44500000000000001</v>
+      </c>
+      <c r="D49" s="42">
+        <f t="shared" si="0"/>
+        <v>0.435</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
+      <c r="B50" s="42">
+        <f t="shared" si="0"/>
+        <v>0.16</v>
+      </c>
+      <c r="C50" s="42">
+        <f t="shared" si="0"/>
+        <v>0.4325</v>
+      </c>
+      <c r="D50" s="42">
+        <f t="shared" si="0"/>
+        <v>0.4325</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
+      <c r="B51" s="42">
+        <f t="shared" si="0"/>
+        <v>0.11000000000000001</v>
+      </c>
+      <c r="C51" s="42">
+        <f t="shared" si="0"/>
+        <v>0.39500000000000002</v>
+      </c>
+      <c r="D51" s="42">
+        <f t="shared" si="0"/>
+        <v>0.41249999999999998</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4">
+      <c r="B52" s="42">
+        <f t="shared" si="0"/>
+        <v>5.2500000000000005E-2</v>
+      </c>
+      <c r="C52" s="42">
+        <f t="shared" si="0"/>
+        <v>0.33499999999999996</v>
+      </c>
+      <c r="D52" s="42">
+        <f t="shared" si="0"/>
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
+      <c r="B53" s="42">
+        <f t="shared" si="0"/>
+        <v>1.5000000000000001E-2</v>
+      </c>
+      <c r="C53" s="42">
+        <f t="shared" si="0"/>
+        <v>0.22499999999999998</v>
+      </c>
+      <c r="D53" s="42">
+        <f t="shared" si="0"/>
+        <v>0.25750000000000001</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
+      <c r="A54" s="40" t="s">
+        <v>37</v>
+      </c>
+      <c r="B54" s="42">
+        <f>SUM(B29:B53)</f>
+        <v>7.2487500000000011</v>
+      </c>
+      <c r="C54" s="42">
+        <f>SUM(C29:C53)</f>
+        <v>10.792499999999999</v>
+      </c>
+      <c r="D54" s="42">
+        <f>SUM(D29:D53)</f>
+        <v>11.054999999999998</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Change website to white-on-black theme
</commit_message>
<xml_diff>
--- a/Voltage_discharge.xlsx
+++ b/Voltage_discharge.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="36" windowWidth="15960" windowHeight="13176" firstSheet="2" activeTab="5"/>
+    <workbookView xWindow="0" yWindow="30" windowWidth="15960" windowHeight="13170" firstSheet="2" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Export Summary" sheetId="1" r:id="rId1"/>
@@ -606,7 +606,7 @@
           <c:x val="9.1001100000000015E-2"/>
           <c:y val="0.12368000000000012"/>
           <c:w val="0.89403199999999949"/>
-          <c:h val="0.81033699999999853"/>
+          <c:h val="0.81033699999999842"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -1879,11 +1879,11 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="165505280"/>
-        <c:axId val="165565952"/>
+        <c:axId val="111181824"/>
+        <c:axId val="111184896"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="165505280"/>
+        <c:axId val="111181824"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1915,14 +1915,14 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="165565952"/>
+        <c:crossAx val="111184896"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
         <c:minorUnit val="0.5"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="165565952"/>
+        <c:axId val="111184896"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="13"/>
@@ -1965,7 +1965,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="165505280"/>
+        <c:crossAx val="111181824"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="0.25"/>
@@ -1989,7 +1989,7 @@
           <c:x val="7.5607700000000014E-2"/>
           <c:y val="0"/>
           <c:w val="0.88914199999999999"/>
-          <c:h val="6.4066700000000185E-2"/>
+          <c:h val="6.4066700000000198E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -2029,7 +2029,7 @@
   </c:spPr>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000133" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000133" header="0.30000000000000032" footer="0.30000000000000032"/>
+    <c:pageMargins b="0.75000000000000144" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000144" header="0.30000000000000032" footer="0.30000000000000032"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -2049,7 +2049,7 @@
           <c:x val="9.1001100000000015E-2"/>
           <c:y val="0.12368000000000012"/>
           <c:w val="0.89403199999999949"/>
-          <c:h val="0.81033699999999853"/>
+          <c:h val="0.81033699999999842"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -3488,11 +3488,11 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="165210752"/>
-        <c:axId val="165228928"/>
+        <c:axId val="110822144"/>
+        <c:axId val="110823680"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="165210752"/>
+        <c:axId val="110822144"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3524,14 +3524,14 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="165228928"/>
+        <c:crossAx val="110823680"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
         <c:minorUnit val="0.5"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="165228928"/>
+        <c:axId val="110823680"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="13"/>
@@ -3574,7 +3574,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="165210752"/>
+        <c:crossAx val="110822144"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="0.25"/>
@@ -3598,7 +3598,7 @@
           <c:x val="7.5607700000000014E-2"/>
           <c:y val="0"/>
           <c:w val="0.88914199999999999"/>
-          <c:h val="6.4066700000000185E-2"/>
+          <c:h val="6.4066700000000198E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -3638,7 +3638,7 @@
   </c:spPr>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000133" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000133" header="0.30000000000000032" footer="0.30000000000000032"/>
+    <c:pageMargins b="0.75000000000000144" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000144" header="0.30000000000000032" footer="0.30000000000000032"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -3655,10 +3655,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="9.1082899999999994E-2"/>
+          <c:x val="9.1082900000000008E-2"/>
           <c:y val="0.12368000000000012"/>
           <c:w val="0.89393599999999951"/>
-          <c:h val="0.81033699999999853"/>
+          <c:h val="0.81033699999999842"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -4600,11 +4600,11 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="165306368"/>
-        <c:axId val="165307904"/>
+        <c:axId val="110880640"/>
+        <c:axId val="110882176"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="165306368"/>
+        <c:axId val="110880640"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4636,14 +4636,14 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="165307904"/>
+        <c:crossAx val="110882176"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="3"/>
         <c:minorUnit val="1.5"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="165307904"/>
+        <c:axId val="110882176"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="13"/>
@@ -4685,7 +4685,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="165306368"/>
+        <c:crossAx val="110880640"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="0.25"/>
@@ -4709,7 +4709,7 @@
           <c:x val="7.5226400000000082E-2"/>
           <c:y val="0"/>
           <c:w val="0.88994100000000065"/>
-          <c:h val="6.4066700000000185E-2"/>
+          <c:h val="6.4066700000000198E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -4749,7 +4749,7 @@
   </c:spPr>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000133" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000133" header="0.30000000000000032" footer="0.30000000000000032"/>
+    <c:pageMargins b="0.75000000000000144" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000144" header="0.30000000000000032" footer="0.30000000000000032"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -4769,7 +4769,7 @@
           <c:x val="9.1001100000000015E-2"/>
           <c:y val="0.12368000000000012"/>
           <c:w val="0.89403199999999949"/>
-          <c:h val="0.81033699999999853"/>
+          <c:h val="0.81033699999999842"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -6042,11 +6042,11 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="165340672"/>
-        <c:axId val="165342208"/>
+        <c:axId val="110960000"/>
+        <c:axId val="110974080"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="165340672"/>
+        <c:axId val="110960000"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6070,7 +6070,7 @@
             <a:pPr>
               <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:schemeClr val="bg1"/>
                 </a:solidFill>
                 <a:latin typeface="Helvetica Neue"/>
               </a:defRPr>
@@ -6078,14 +6078,14 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="165342208"/>
+        <c:crossAx val="110974080"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
         <c:minorUnit val="0.5"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="165342208"/>
+        <c:axId val="110974080"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="13"/>
@@ -6120,7 +6120,7 @@
             <a:pPr>
               <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:schemeClr val="bg1"/>
                 </a:solidFill>
                 <a:latin typeface="Helvetica Neue"/>
               </a:defRPr>
@@ -6128,7 +6128,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="165340672"/>
+        <c:crossAx val="110960000"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="0.25"/>
@@ -6145,6 +6145,42 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="t"/>
+      <c:legendEntry>
+        <c:idx val="0"/>
+        <c:txPr>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:schemeClr val="bg1"/>
+                </a:solidFill>
+                <a:latin typeface="Helvetica Neue"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+      </c:legendEntry>
+      <c:legendEntry>
+        <c:idx val="1"/>
+        <c:txPr>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:schemeClr val="bg1"/>
+                </a:solidFill>
+                <a:latin typeface="Helvetica Neue"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+      </c:legendEntry>
       <c:layout>
         <c:manualLayout>
           <c:xMode val="edge"/>
@@ -6152,14 +6188,16 @@
           <c:x val="7.5607700000000014E-2"/>
           <c:y val="0"/>
           <c:w val="0.88914199999999999"/>
-          <c:h val="6.4066700000000185E-2"/>
+          <c:h val="6.4066700000000198E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
       <c:spPr>
         <a:noFill/>
         <a:ln w="12700" cap="flat">
-          <a:noFill/>
+          <a:solidFill>
+            <a:schemeClr val="bg1"/>
+          </a:solidFill>
           <a:miter lim="400000"/>
         </a:ln>
         <a:effectLst/>
@@ -6184,7 +6222,9 @@
     <c:dispBlanksAs val="gap"/>
   </c:chart>
   <c:spPr>
-    <a:noFill/>
+    <a:solidFill>
+      <a:schemeClr val="tx1"/>
+    </a:solidFill>
     <a:ln>
       <a:noFill/>
     </a:ln>
@@ -6192,7 +6232,7 @@
   </c:spPr>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000133" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000133" header="0.30000000000000032" footer="0.30000000000000032"/>
+    <c:pageMargins b="0.75000000000000144" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000144" header="0.30000000000000032" footer="0.30000000000000032"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -6209,10 +6249,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="6.4312400000000242E-2"/>
+          <c:x val="6.4312400000000269E-2"/>
           <c:y val="0.12368000000000012"/>
           <c:w val="0.88765000000000005"/>
-          <c:h val="0.81033699999999853"/>
+          <c:h val="0.81033699999999842"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -6420,11 +6460,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="165501568"/>
-        <c:axId val="165527936"/>
+        <c:axId val="110998272"/>
+        <c:axId val="110999808"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="165501568"/>
+        <c:axId val="110998272"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="806395000"/>
@@ -6457,12 +6497,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="165527936"/>
+        <c:crossAx val="110999808"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="165527936"/>
+        <c:axId val="110999808"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6503,7 +6543,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="165501568"/>
+        <c:crossAx val="110998272"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="0.2"/>
@@ -6527,7 +6567,7 @@
           <c:x val="4.0081200000000004E-2"/>
           <c:y val="0"/>
           <c:w val="0.9"/>
-          <c:h val="6.4066700000000185E-2"/>
+          <c:h val="6.4066700000000198E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -6567,7 +6607,7 @@
   </c:spPr>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000133" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000133" header="0.30000000000000032" footer="0.30000000000000032"/>
+    <c:pageMargins b="0.75000000000000144" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000144" header="0.30000000000000032" footer="0.30000000000000032"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -7181,11 +7221,11 @@
           </c:val>
         </c:ser>
         <c:marker val="1"/>
-        <c:axId val="165717504"/>
-        <c:axId val="165719040"/>
+        <c:axId val="111204224"/>
+        <c:axId val="111205760"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="165717504"/>
+        <c:axId val="111204224"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7193,14 +7233,14 @@
         <c:numFmt formatCode="h:mm\ AM/PM" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="165719040"/>
+        <c:crossAx val="111205760"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="165719040"/>
+        <c:axId val="111205760"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7227,7 +7267,7 @@
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="165717504"/>
+        <c:crossAx val="111204224"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7240,7 +7280,7 @@
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000089" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000089" header="0.30000000000000032" footer="0.30000000000000032"/>
+    <c:pageMargins b="0.750000000000001" l="0.70000000000000062" r="0.70000000000000062" t="0.750000000000001" header="0.30000000000000032" footer="0.30000000000000032"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -8489,20 +8529,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="B3:D16"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="13.05" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="13.15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
-    <col min="2" max="4" width="33.5546875" customWidth="1"/>
+    <col min="2" max="4" width="33.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:4" ht="49.95" customHeight="1">
+    <row r="3" spans="2:4" ht="49.9" customHeight="1">
       <c r="B3" s="46" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="47"/>
       <c r="D3" s="47"/>
     </row>
-    <row r="7" spans="2:4" ht="17.399999999999999">
+    <row r="7" spans="2:4" ht="18">
       <c r="B7" s="1" t="s">
         <v>1</v>
       </c>
@@ -8594,10 +8634,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I263"/>
-  <sheetFormatPr defaultColWidth="16.33203125" defaultRowHeight="19.95" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="16.28515625" defaultRowHeight="19.899999999999999" customHeight="1"/>
   <cols>
-    <col min="1" max="10" width="16.33203125" style="5" customWidth="1"/>
-    <col min="11" max="16384" width="16.33203125" style="5"/>
+    <col min="1" max="10" width="16.28515625" style="5" customWidth="1"/>
+    <col min="11" max="16384" width="16.28515625" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="27.75" customHeight="1">
@@ -8613,7 +8653,7 @@
       <c r="H1" s="48"/>
       <c r="I1" s="48"/>
     </row>
-    <row r="2" spans="1:9" ht="20.55" customHeight="1">
+    <row r="2" spans="1:9" ht="20.65" customHeight="1">
       <c r="A2" s="6"/>
       <c r="B2" s="6"/>
       <c r="C2" s="7" t="s">
@@ -12769,10 +12809,10 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G263"/>
-  <sheetFormatPr defaultColWidth="16.33203125" defaultRowHeight="19.95" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="16.28515625" defaultRowHeight="19.899999999999999" customHeight="1"/>
   <cols>
-    <col min="1" max="8" width="16.33203125" style="19" customWidth="1"/>
-    <col min="9" max="16384" width="16.33203125" style="19"/>
+    <col min="1" max="8" width="16.28515625" style="19" customWidth="1"/>
+    <col min="9" max="16384" width="16.28515625" style="19"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="27.75" customHeight="1">
@@ -12786,7 +12826,7 @@
       <c r="F1" s="48"/>
       <c r="G1" s="48"/>
     </row>
-    <row r="2" spans="1:7" ht="20.55" customHeight="1">
+    <row r="2" spans="1:7" ht="20.65" customHeight="1">
       <c r="A2" s="6"/>
       <c r="B2" s="6"/>
       <c r="C2" s="7" t="s">
@@ -16640,12 +16680,12 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G33"/>
-  <sheetFormatPr defaultColWidth="16.33203125" defaultRowHeight="19.95" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="16.28515625" defaultRowHeight="19.899999999999999" customHeight="1"/>
   <cols>
-    <col min="1" max="5" width="16.33203125" style="20" customWidth="1"/>
-    <col min="6" max="6" width="22.21875" style="20" customWidth="1"/>
-    <col min="7" max="8" width="16.33203125" style="20" customWidth="1"/>
-    <col min="9" max="16384" width="16.33203125" style="20"/>
+    <col min="1" max="5" width="16.28515625" style="20" customWidth="1"/>
+    <col min="6" max="6" width="22.28515625" style="20" customWidth="1"/>
+    <col min="7" max="8" width="16.28515625" style="20" customWidth="1"/>
+    <col min="9" max="16384" width="16.28515625" style="20"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="27.75" customHeight="1">
@@ -16659,7 +16699,7 @@
       <c r="F1" s="48"/>
       <c r="G1" s="48"/>
     </row>
-    <row r="2" spans="1:7" ht="20.55" customHeight="1">
+    <row r="2" spans="1:7" ht="20.65" customHeight="1">
       <c r="A2" s="21"/>
       <c r="B2" s="7" t="s">
         <v>18</v>
@@ -16676,7 +16716,7 @@
       <c r="F2" s="21"/>
       <c r="G2" s="21"/>
     </row>
-    <row r="3" spans="1:7" ht="20.55" customHeight="1">
+    <row r="3" spans="1:7" ht="20.65" customHeight="1">
       <c r="A3" s="22"/>
       <c r="B3" s="23">
         <v>46225.28125</v>
@@ -16696,7 +16736,7 @@
       </c>
       <c r="G3" s="30"/>
     </row>
-    <row r="4" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="4" spans="1:7" ht="20.45" customHeight="1">
       <c r="A4" s="27"/>
       <c r="B4" s="28">
         <v>46225.302083333336</v>
@@ -16717,7 +16757,7 @@
         <v>0.17249999999999996</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="5" spans="1:7" ht="20.45" customHeight="1">
       <c r="A5" s="27"/>
       <c r="B5" s="28">
         <v>46225.322916666664</v>
@@ -16738,7 +16778,7 @@
         <v>0.19999999999999998</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="6" spans="1:7" ht="20.45" customHeight="1">
       <c r="A6" s="13"/>
       <c r="B6" s="28">
         <v>46225.34375</v>
@@ -16759,7 +16799,7 @@
         <v>0.19500000000000003</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="7" spans="1:7" ht="20.45" customHeight="1">
       <c r="A7" s="13"/>
       <c r="B7" s="28">
         <v>46225.364583333336</v>
@@ -16780,7 +16820,7 @@
         <v>0.16750000000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="8" spans="1:7" ht="20.45" customHeight="1">
       <c r="A8" s="27"/>
       <c r="B8" s="28">
         <v>46225.385416666664</v>
@@ -16801,7 +16841,7 @@
         <v>0.125</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="9" spans="1:7" ht="20.45" customHeight="1">
       <c r="A9" s="27"/>
       <c r="B9" s="31">
         <v>46225.385416666664</v>
@@ -16814,7 +16854,7 @@
       <c r="F9" s="30"/>
       <c r="G9" s="30"/>
     </row>
-    <row r="10" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="10" spans="1:7" ht="20.45" customHeight="1">
       <c r="A10" s="27"/>
       <c r="B10" s="28">
         <v>46225.40625</v>
@@ -16835,7 +16875,7 @@
         <v>8.500000000000002E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="11" spans="1:7" ht="20.45" customHeight="1">
       <c r="A11" s="27"/>
       <c r="B11" s="28">
         <v>46225.427083333336</v>
@@ -16856,7 +16896,7 @@
         <v>5.7500000000000051E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="12" spans="1:7" ht="20.45" customHeight="1">
       <c r="A12" s="27"/>
       <c r="B12" s="28">
         <v>46225.447916666664</v>
@@ -16877,7 +16917,7 @@
         <v>3.0000000000000027E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="13" spans="1:7" ht="20.45" customHeight="1">
       <c r="A13" s="27"/>
       <c r="B13" s="28">
         <v>46225.46875</v>
@@ -16898,7 +16938,7 @@
         <v>5.00000000000006E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="14" spans="1:7" ht="20.45" customHeight="1">
       <c r="A14" s="27"/>
       <c r="B14" s="28">
         <v>46225.489583333336</v>
@@ -16919,7 +16959,7 @@
         <v>-1.4999999999999958E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="15" spans="1:7" ht="20.45" customHeight="1">
       <c r="A15" s="27"/>
       <c r="B15" s="28">
         <v>46225.510416666664</v>
@@ -16940,7 +16980,7 @@
         <v>-2.4999999999999967E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="16" spans="1:7" ht="20.45" customHeight="1">
       <c r="A16" s="27"/>
       <c r="B16" s="28">
         <v>46225.53125</v>
@@ -16961,7 +17001,7 @@
         <v>-3.2499999999999973E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="17" spans="1:7" ht="20.45" customHeight="1">
       <c r="A17" s="27"/>
       <c r="B17" s="28">
         <v>46225.552083333336</v>
@@ -16982,7 +17022,7 @@
         <v>-3.2499999999999973E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="18" spans="1:7" ht="20.45" customHeight="1">
       <c r="A18" s="27"/>
       <c r="B18" s="28">
         <v>46225.572916666664</v>
@@ -17003,7 +17043,7 @@
         <v>-2.9999999999999971E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="19" spans="1:7" ht="20.45" customHeight="1">
       <c r="A19" s="27"/>
       <c r="B19" s="28">
         <v>46225.59375</v>
@@ -17024,7 +17064,7 @@
         <v>-1.9999999999999962E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="20" spans="1:7" ht="20.45" customHeight="1">
       <c r="A20" s="27"/>
       <c r="B20" s="28">
         <v>46225.614583333336</v>
@@ -17045,7 +17085,7 @@
         <v>-5.0000000000000044E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="21" spans="1:7" ht="20.45" customHeight="1">
       <c r="A21" s="27"/>
       <c r="B21" s="28">
         <v>46225.635416666664</v>
@@ -17066,7 +17106,7 @@
         <v>7.5000000000000067E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="22" spans="1:7" ht="20.45" customHeight="1">
       <c r="A22" s="27"/>
       <c r="B22" s="28">
         <v>46225.65625</v>
@@ -17087,7 +17127,7 @@
         <v>3.0000000000000027E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="23" spans="1:7" ht="20.45" customHeight="1">
       <c r="A23" s="27"/>
       <c r="B23" s="28">
         <v>46225.677083333336</v>
@@ -17108,7 +17148,7 @@
         <v>6.5000000000000058E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="24" spans="1:7" ht="20.45" customHeight="1">
       <c r="A24" s="27"/>
       <c r="B24" s="28">
         <v>46225.697916666664</v>
@@ -17129,7 +17169,7 @@
         <v>9.9999999999999978E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="25" spans="1:7" ht="20.45" customHeight="1">
       <c r="A25" s="27"/>
       <c r="B25" s="28">
         <v>46225.697916666664</v>
@@ -17142,7 +17182,7 @@
       <c r="F25" s="30"/>
       <c r="G25" s="30"/>
     </row>
-    <row r="26" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="26" spans="1:7" ht="20.45" customHeight="1">
       <c r="A26" s="27"/>
       <c r="B26" s="28">
         <v>46225.71875</v>
@@ -17163,7 +17203,7 @@
         <v>0.11000000000000004</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="27" spans="1:7" ht="20.45" customHeight="1">
       <c r="A27" s="27"/>
       <c r="B27" s="28">
         <v>46225.739583333336</v>
@@ -17184,7 +17224,7 @@
         <v>0.15750000000000003</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="28" spans="1:7" ht="20.45" customHeight="1">
       <c r="A28" s="27"/>
       <c r="B28" s="28">
         <v>46225.760416666664</v>
@@ -17205,7 +17245,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="29" spans="1:7" ht="20.45" customHeight="1">
       <c r="A29" s="32" t="s">
         <v>21</v>
       </c>
@@ -17220,7 +17260,7 @@
       <c r="F29" s="30"/>
       <c r="G29" s="30"/>
     </row>
-    <row r="30" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="30" spans="1:7" ht="20.45" customHeight="1">
       <c r="A30" s="32" t="s">
         <v>22</v>
       </c>
@@ -17235,7 +17275,7 @@
       <c r="F30" s="30"/>
       <c r="G30" s="30"/>
     </row>
-    <row r="31" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="31" spans="1:7" ht="20.45" customHeight="1">
       <c r="A31" s="34" t="s">
         <v>23</v>
       </c>
@@ -17251,7 +17291,7 @@
         <v>1.5475000000000005</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="20.399999999999999" customHeight="1">
+    <row r="32" spans="1:7" ht="20.45" customHeight="1">
       <c r="A32" s="32" t="s">
         <v>24</v>
       </c>
@@ -17268,7 +17308,7 @@
         <v>2.4141666666666675</v>
       </c>
     </row>
-    <row r="33" spans="7:7" ht="19.95" customHeight="1">
+    <row r="33" spans="7:7" ht="19.899999999999999" customHeight="1">
       <c r="G33" s="20">
         <f>G32/'Riemann Sum - Midpoint Riemann '!I31</f>
         <v>0.31702779601663394</v>
@@ -17293,10 +17333,10 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I34"/>
-  <sheetFormatPr defaultColWidth="16.33203125" defaultRowHeight="19.95" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="16.28515625" defaultRowHeight="19.899999999999999" customHeight="1"/>
   <cols>
-    <col min="1" max="10" width="16.33203125" style="35" customWidth="1"/>
-    <col min="11" max="16384" width="16.33203125" style="35"/>
+    <col min="1" max="10" width="16.28515625" style="35" customWidth="1"/>
+    <col min="11" max="16384" width="16.28515625" style="35"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="27.75" customHeight="1">
@@ -17339,7 +17379,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="20.55" customHeight="1">
+    <row r="3" spans="1:9" ht="20.65" customHeight="1">
       <c r="A3" s="23">
         <v>46225.28125</v>
       </c>
@@ -17362,7 +17402,7 @@
       </c>
       <c r="I3" s="12"/>
     </row>
-    <row r="4" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="4" spans="1:9" ht="20.45" customHeight="1">
       <c r="A4" s="28">
         <v>46225.302083333336</v>
       </c>
@@ -17386,7 +17426,7 @@
         <v>2.4999999999999994E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="5" spans="1:9" ht="20.45" customHeight="1">
       <c r="A5" s="28">
         <v>46225.322916666664</v>
       </c>
@@ -17458,7 +17498,7 @@
         <v>0.19749999999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="8" spans="1:9" ht="20.45" customHeight="1">
       <c r="A8" s="28">
         <v>46225.385416666664</v>
       </c>
@@ -17482,7 +17522,7 @@
         <v>0.255</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="9" spans="1:9" ht="20.45" customHeight="1">
       <c r="A9" s="31">
         <v>46225.385416666664</v>
       </c>
@@ -17500,7 +17540,7 @@
       </c>
       <c r="I9" s="16"/>
     </row>
-    <row r="10" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="10" spans="1:9" ht="20.45" customHeight="1">
       <c r="A10" s="28">
         <v>46225.40625</v>
       </c>
@@ -17524,7 +17564,7 @@
         <v>0.3125</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="11" spans="1:9" ht="20.45" customHeight="1">
       <c r="A11" s="28">
         <v>46225.427083333336</v>
       </c>
@@ -17548,7 +17588,7 @@
         <v>0.35499999999999998</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="12" spans="1:9" ht="20.45" customHeight="1">
       <c r="A12" s="28">
         <v>46225.447916666664</v>
       </c>
@@ -17572,7 +17612,7 @@
         <v>0.39750000000000002</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="13" spans="1:9" ht="20.45" customHeight="1">
       <c r="A13" s="28">
         <v>46225.46875</v>
       </c>
@@ -17596,7 +17636,7 @@
         <v>0.4325</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="14" spans="1:9" ht="20.45" customHeight="1">
       <c r="A14" s="28">
         <v>46225.489583333336</v>
       </c>
@@ -17620,7 +17660,7 @@
         <v>0.46</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="15" spans="1:9" ht="20.45" customHeight="1">
       <c r="A15" s="28">
         <v>46225.510416666664</v>
       </c>
@@ -17644,7 +17684,7 @@
         <v>0.47499999999999998</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="16" spans="1:9" ht="20.45" customHeight="1">
       <c r="A16" s="28">
         <v>46225.53125</v>
       </c>
@@ -17668,7 +17708,7 @@
         <v>0.48499999999999999</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="17" spans="1:9" ht="20.45" customHeight="1">
       <c r="A17" s="28">
         <v>46225.552083333336</v>
       </c>
@@ -17692,7 +17732,7 @@
         <v>0.48749999999999999</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="18" spans="1:9" ht="20.45" customHeight="1">
       <c r="A18" s="28">
         <v>46225.572916666664</v>
       </c>
@@ -17716,7 +17756,7 @@
         <v>0.48249999999999998</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="19" spans="1:9" ht="20.45" customHeight="1">
       <c r="A19" s="28">
         <v>46225.59375</v>
       </c>
@@ -17740,7 +17780,7 @@
         <v>0.47</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="20" spans="1:9" ht="20.45" customHeight="1">
       <c r="A20" s="28">
         <v>46225.614583333336</v>
       </c>
@@ -17764,7 +17804,7 @@
         <v>0.45000000000000007</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="21" spans="1:9" ht="20.45" customHeight="1">
       <c r="A21" s="28">
         <v>46225.635416666664</v>
       </c>
@@ -17788,7 +17828,7 @@
         <v>0.42750000000000005</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="22" spans="1:9" ht="20.45" customHeight="1">
       <c r="A22" s="28">
         <v>46225.65625</v>
       </c>
@@ -17812,7 +17852,7 @@
         <v>0.39500000000000002</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="23" spans="1:9" ht="20.45" customHeight="1">
       <c r="A23" s="28">
         <v>46225.677083333336</v>
       </c>
@@ -17836,7 +17876,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="24" spans="1:9" ht="20.45" customHeight="1">
       <c r="A24" s="28">
         <v>46225.697916666664</v>
       </c>
@@ -17860,7 +17900,7 @@
         <v>0.30000000000000004</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="25" spans="1:9" ht="20.45" customHeight="1">
       <c r="A25" s="28">
         <v>46225.697916666664</v>
       </c>
@@ -17878,7 +17918,7 @@
       </c>
       <c r="I25" s="16"/>
     </row>
-    <row r="26" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="26" spans="1:9" ht="20.45" customHeight="1">
       <c r="A26" s="28">
         <v>46225.71875</v>
       </c>
@@ -17902,7 +17942,7 @@
         <v>0.26999999999999996</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="27" spans="1:9" ht="20.45" customHeight="1">
       <c r="A27" s="28">
         <v>46225.739583333336</v>
       </c>
@@ -17926,7 +17966,7 @@
         <v>0.21499999999999997</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="28" spans="1:9" ht="20.45" customHeight="1">
       <c r="A28" s="28">
         <v>46225.760416666664</v>
       </c>
@@ -17950,7 +17990,7 @@
         <v>0.15249999999999997</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="29" spans="1:9" ht="20.45" customHeight="1">
       <c r="A29" s="28">
         <v>0.78125</v>
       </c>
@@ -17963,7 +18003,7 @@
       <c r="H29" s="15"/>
       <c r="I29" s="15"/>
     </row>
-    <row r="30" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="30" spans="1:9" ht="20.45" customHeight="1">
       <c r="A30" s="28">
         <v>0.80208333333333337</v>
       </c>
@@ -17976,7 +18016,7 @@
       <c r="H30" s="15"/>
       <c r="I30" s="15"/>
     </row>
-    <row r="31" spans="1:9" ht="20.399999999999999" customHeight="1">
+    <row r="31" spans="1:9" ht="20.45" customHeight="1">
       <c r="A31" s="33"/>
       <c r="B31" s="33"/>
       <c r="C31" s="15" cm="1">
@@ -17993,13 +18033,13 @@
         <v>7.6149999999999993</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="19.95" customHeight="1">
+    <row r="32" spans="1:9" ht="19.899999999999999" customHeight="1">
       <c r="A32" s="33"/>
     </row>
-    <row r="33" spans="1:1" ht="19.95" customHeight="1">
+    <row r="33" spans="1:1" ht="19.899999999999999" customHeight="1">
       <c r="A33" s="14"/>
     </row>
-    <row r="34" spans="1:1" ht="19.95" customHeight="1">
+    <row r="34" spans="1:1" ht="19.899999999999999" customHeight="1">
       <c r="A34" s="33"/>
     </row>
   </sheetData>
@@ -18017,15 +18057,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E54"/>
-  <sheetFormatPr defaultRowHeight="13.2"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="1" width="14.77734375" style="42" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" style="42" customWidth="1"/>
     <col min="2" max="2" width="13" style="42" customWidth="1"/>
-    <col min="3" max="3" width="11.109375" style="42" customWidth="1"/>
-    <col min="4" max="4" width="9.109375" style="42"/>
+    <col min="3" max="3" width="11.140625" style="42" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" style="42"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="24.6">
+    <row r="1" spans="1:5" ht="24.75">
       <c r="A1" s="44" t="s">
         <v>18</v>
       </c>

</xml_diff>